<commit_message>
Comissão de parceiros: 3 quick wins grátis, menção ao nosso nome e 15% de cada trabalho recomendado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bCka4TNe6PKPBEx4M62DX
</commit_message>
<xml_diff>
--- a/research/instagram/prospecao-instagram.xlsx
+++ b/research/instagram/prospecao-instagram.xlsx
@@ -725,12 +725,12 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>DM personalizada a pedir uma conversa curta para mostrar o Partner Systems Opportunity Map.</t>
+          <t>DM personalizada a oferecer 3 soluções rápidas implementadas sem custo, a partir do mapa da operação dele.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Conversa curta → entregar o mapa → confiança → introduções consentidas a negócios com gargalo operacional.</t>
+          <t>Conversa → 3 quick wins implementados → mostram o nosso nome por gratidão → recomendam, com 15% de cada trabalho que vier deles.</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
@@ -833,12 +833,12 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>DM personalizada a pedir uma conversa curta para mostrar o Partner Systems Opportunity Map.</t>
+          <t>DM personalizada a oferecer 3 soluções rápidas implementadas sem custo, a partir do mapa da operação dele.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Conversa curta → entregar o mapa → confiança → introduções consentidas a negócios com gargalo operacional.</t>
+          <t>Conversa → 3 quick wins implementados → mostram o nosso nome por gratidão → recomendam, com 15% de cada trabalho que vier deles.</t>
         </is>
       </c>
       <c r="O3" s="2" t="n">
@@ -941,12 +941,12 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>DM personalizada a pedir uma conversa curta para mostrar o Partner Systems Opportunity Map.</t>
+          <t>DM personalizada a oferecer 3 soluções rápidas implementadas sem custo, a partir do mapa da operação dele.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Conversa curta → entregar o mapa → confiança → introduções consentidas a negócios com gargalo operacional.</t>
+          <t>Conversa → 3 quick wins implementados → mostram o nosso nome por gratidão → recomendam, com 15% de cada trabalho que vier deles.</t>
         </is>
       </c>
       <c r="O4" s="2" t="n">
@@ -1053,12 +1053,12 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>DM personalizada a pedir uma conversa curta para mostrar o Partner Systems Opportunity Map.</t>
+          <t>DM personalizada a oferecer 3 soluções rápidas implementadas sem custo, a partir do mapa da operação dele.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Conversa curta → entregar o mapa → confiança → introduções consentidas a negócios com gargalo operacional.</t>
+          <t>Conversa → 3 quick wins implementados → mostram o nosso nome por gratidão → recomendam, com 15% de cada trabalho que vier deles.</t>
         </is>
       </c>
       <c r="O5" s="2" t="n">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Co-entrega, introdução mútua ou workshop; referrals qualificados e casos partilháveis.</t>
+          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
         </is>
       </c>
       <c r="O7" s="2" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Co-entrega, introdução mútua ou workshop; referrals qualificados e casos partilháveis.</t>
+          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
         </is>
       </c>
       <c r="O8" s="2" t="n">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Co-entrega, introdução mútua ou workshop; referrals qualificados e casos partilháveis.</t>
+          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
         </is>
       </c>
       <c r="O9" s="2" t="n">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Co-entrega, introdução mútua ou workshop; referrals qualificados e casos partilháveis.</t>
+          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
         </is>
       </c>
       <c r="O10" s="2" t="n">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Co-entrega, introdução mútua ou workshop; referrals qualificados e casos partilháveis.</t>
+          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
         </is>
       </c>
       <c r="O11" s="2" t="n">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Co-entrega, introdução mútua ou workshop; referrals qualificados e casos partilháveis.</t>
+          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
         </is>
       </c>
       <c r="O12" s="2" t="n">
@@ -7171,17 +7171,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>DM personalizada a pedir uma conversa curta para mostrar o Partner Systems Opportunity Map.</t>
+          <t>DM personalizada a oferecer 3 soluções rápidas implementadas sem custo, a partir do mapa da operação dele.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Partner Systems Opportunity Map: 3 a 5 handoffs, uma hipótese de melhoria, um limite humano e uma prioridade de 30 dias.</t>
+          <t>3 quick wins implementados sem custo, escolhidos pela situação atual (mapa com 3 a 5 handoffs como base).</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Conversa curta → entregar o mapa → confiança → introduções consentidas a negócios com gargalo operacional.</t>
+          <t>Conversa → 3 quick wins implementados → mostram o nosso nome por gratidão → recomendam, com 15% de cada trabalho que vier deles.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -7250,12 +7250,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mini-mapa de um fluxo conjunto ou de um cliente-tipo da agência.</t>
+          <t>3 quick wins implementados sem custo na operação da agência; mini-mapa de um cliente-tipo.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Co-entrega, introdução mútua ou workshop; referrals qualificados e casos partilháveis.</t>
+          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7361,7 +7361,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho} și m-am gândit la partea din spate a operațiunii tale: {percurso}. Am pregătit ceva util pentru tine, fără cost: o hartă scurtă cu 3–5 predări între oameni și sisteme, o ipoteză de îmbunătățire, punctul unde decide un om și prioritatea pentru următoarele 30 de zile. Întrebarea de la care pornesc: {pergunta} Ai fi deschis la o scurtă întâlnire ca să ți-o arăt? Voi fi pregătit.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho} și m-am gândit la partea din spate a operațiunii tale: {percurso}. Vreau să-ți ofer ceva concret, fără cost: pornind de la situația ta de acum, implementăm 3 soluții rapide în operațiunea ta. Întrebarea de la care pornesc: {pergunta} Ai fi deschis la o scurtă întâlnire ca să alegem împreună cele 3 soluții? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin pe scurt, cu un lucru concret: {valor} Harta rămâne pregătită pentru tine, fără nicio obligație. Dacă acum nu e momentul, înțeleg perfect. Voi fi pregătit.</t>
+          <t>{saudacao} Revin pe scurt, cu un lucru concret: {valor} Oferta celor 3 soluții rămâne valabilă, fără nicio obligație. Dacă acum nu e momentul, înțeleg perfect. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7395,17 +7395,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho} e fiquei a pensar na parte de trás da tua operação: {percurso}. Preparei uma coisa útil para ti, sem custo: um mapa curto com 3 a 5 passagens entre pessoas e sistemas, uma hipótese de melhoria, o ponto onde decide uma pessoa e a prioridade para os próximos 30 dias. A pergunta de onde parto: {pergunta} Estarias aberto a uma conversa curta para te mostrar? Vou estar preparado.</t>
+          <t>{saudacao} Mă bucur că cele 3 soluții merg deja la tine. Am o propunere simplă de parteneriat. Dacă ți se pare corect, menționează Pacheco Studios ca pe cei care te-au ajutat: o postare sau un story cu @pachecostudiospt și un rând pe site. Apoi, când întâlnești o afacere care se blochează în același loc, ne faci o introducere, cu acordul ei. Pentru fiecare lucrare care vine din recomandarea ta primești 15% din valoarea ei, plătit în 7 zile de la plata clientului. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7422,12 +7422,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto só com uma coisa concreta: {valor} O mapa continua preparado para ti, sem compromisso. Se agora não é o momento, percebo perfeitamente. Vou estar preparado.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho} e fiquei a pensar na parte de trás da tua operação: {percurso}. Quero oferecer-te uma coisa concreta, sem custo: a partir da tua situação atual, implementamos 3 soluções rápidas na tua operação. A pergunta de onde parto: {pergunta} Estarias aberto a uma conversa curta para escolhermos juntos as 3 soluções? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7439,17 +7439,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho} and started thinking about the back end of your operation: {percurso}. I put together something useful for you, at no cost: a short map with 3 to 5 handoffs between people and systems, one improvement hypothesis, the point where a human decides, and a 30-day priority. The question I start from: {pergunta} Would you be open to a short call so I can walk you through it? I'll come prepared.</t>
+          <t>{saudacao} Volto só com uma coisa concreta: {valor} A oferta das 3 soluções mantém-se, sem compromisso. Se agora não é o momento, percebo perfeitamente. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7461,29 +7461,29 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} A quick follow-up with one concrete thing: {valor} The map is still ready for you, no strings attached. If now isn't the right time, completely understood. I'll come prepared.</t>
+          <t>{saudacao} Fico contente por as 3 soluções já estarem a funcionar contigo. Tenho uma proposta simples de parceria. Se te parecer justo, menciona a Pacheco Studios como quem te ajudou: um post ou story com @pachecostudiospt e uma linha no site. Depois, quando conheceres um negócio que encrava no mesmo sítio, apresentas-nos, com o acordo dele. Por cada trabalho que vier da tua recomendação recebes 15% do valor, pago até 7 dias depois de o cliente pagar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Grande negócio</t>
+          <t>Influenciador / operador</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -7493,19 +7493,19 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am parcurs traseul public al unui client {empresa}: {percurso}. Pe baza a ceea ce este public, am o ipoteză de diagnostic, nu o concluzie: {pergunta} Am pus-o pe o mini-hartă de o pagină. Cu cine din echipă ar fi potrivit să o validez: operațiuni, experiența clienților sau transformare digitală? O întâlnire scurtă de explorare ar fi suficientă. Voi fi pregătit.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho} and started thinking about the back end of your operation: {percurso}. I'd like to offer you something concrete, at no cost: based on where your operation is today, we implement 3 quick wins in it. The question I start from: {pergunta} Would you be open to a short call to pick the 3 together? I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Grande negócio</t>
+          <t>Influenciador / operador</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -7515,29 +7515,29 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu mini-harta despre traseul clientului {empresa}. Am adăugat un singur punct: {valor} Dacă îmi puteți indica persoana potrivită, îi trimit direct harta. Voi fi pregătit.</t>
+          <t>{saudacao} A quick follow-up with one concrete thing: {valor} The offer of the 3 quick wins still stands, no strings attached. If now isn't the right time, completely understood. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Grande negócio</t>
+          <t>Influenciador / operador</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Percorri o percurso público de um cliente {empresa}: {percurso}. Com base no que é público, tenho uma hipótese de diagnóstico, não uma conclusão: {pergunta} Pus isto num mini-mapa de uma página. Quem na equipa seria a pessoa certa para o validar: operações, experiência do cliente ou transformação digital? Uma conversa exploratória curta chega. Vou estar preparado.</t>
+          <t>{saudacao} Glad the 3 quick wins are already working for you. I have a simple partnership proposal. If it feels fair, mention Pacheco Studios as the team that helped you: a post or story tagging @pachecostudiospt and a line on your site. Then, when you meet a business stuck in the same place, introduce us, with their consent. For every job that comes from your referral you get 15% of its value, paid within 7 days of the client paying. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -7549,17 +7549,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto ao mini-mapa sobre o percurso do cliente {empresa}. Acrescentei um único ponto: {valor} Se me puderem indicar a pessoa certa, envio-lhe o mapa diretamente. Vou estar preparado.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am parcurs traseul public al unui client {empresa}: {percurso}. Pe baza a ceea ce este public, am o ipoteză de diagnostic, nu o concluzie: {pergunta} Am pus-o pe o mini-hartă de o pagină. Cu cine din echipă ar fi potrivit să o validez: operațiuni, experiența clienților sau transformare digitală? O întâlnire scurtă de explorare ar fi suficientă. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7571,17 +7571,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I walked through the public journey of a {empresa} customer: {percurso}. Based only on what's public, I have a diagnostic hypothesis, not a conclusion: {pergunta} I've put it on a one-page mini-map. Who on the team would be the right person to validate it: operations, customer experience or digital transformation? A short exploratory call would be enough. I'll come prepared.</t>
+          <t>{saudacao} Revin cu mini-harta despre traseul clientului {empresa}. Am adăugat un singur punct: {valor} Dacă îmi puteți indica persoana potrivită, îi trimit direct harta. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7593,83 +7593,83 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Following up on the mini-map of the {empresa} customer journey. I added one point: {valor} If you can point me to the right person, I'll send the map to them directly. I'll come prepared.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Percorri o percurso público de um cliente {empresa}: {percurso}. Com base no que é público, tenho uma hipótese de diagnóstico, não uma conclusão: {pergunta} Pus isto num mini-mapa de uma página. Quem na equipa seria a pessoa certa para o validar: operações, experiência do cliente ou transformação digital? Uma conversa exploratória curta chega. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho}. Voi aduceți cererea; noi lucrăm în stratul de după lead: cum ajunge cererea la echipă, ce context o însoțește, cine decide și cum se livrează. Nu înlocuim marketingul sau brandingul, protejăm rezultatul pe care îl generați deja. Am schițat o mini-hartă pentru un client tipic de-al vostru: {percurso}. Ați fi deschis la o întâlnire ca să vedem dacă are sens să lucrăm împreună? Voi fi pregătit.</t>
+          <t>{saudacao} Volto ao mini-mapa sobre o percurso do cliente {empresa}. Acrescentei um único ponto: {valor} Se me puderem indicar a pessoa certa, envio-lhe o mapa diretamente. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu un exemplu concret de colaborare: {valor} Voi păstrați relația și serviciul, noi intrăm doar pe partea operațională. Voi fi pregătit.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I walked through the public journey of a {empresa} customer: {percurso}. Based only on what's public, I have a diagnostic hypothesis, not a conclusion: {pergunta} I've put it on a one-page mini-map. Who on the team would be the right person to validate it: operations, customer experience or digital transformation? A short exploratory call would be enough. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho}. Vocês trazem a procura; nós trabalhamos na camada depois do lead: como o pedido chega à equipa, que contexto leva, quem decide e como se entrega. Não substituímos o marketing nem a marca, protegemos o resultado que vocês já geram. Esbocei um mini-mapa para um cliente típico vosso: {percurso}. Estariam abertos a uma reunião para ver se faz sentido trabalharmos juntos? Vou estar preparado.</t>
+          <t>{saudacao} Following up on the mini-map of the {empresa} customer journey. I added one point: {valor} If you can point me to the right person, I'll send the map to them directly. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -7681,17 +7681,17 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto com um exemplo concreto de colaboração: {valor} Vocês mantêm a relação e o serviço, nós entramos só na parte operacional. Vou estar preparado.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho}. Voi aduceți cererea; noi lucrăm în stratul de după lead: cum ajunge cererea la echipă, ce context o însoțește, cine decide și cum se livrează. Nu înlocuim marketingul sau brandingul, protejăm rezultatul pe care îl generați deja. Am schițat o mini-hartă pentru un client tipic de-al vostru: {percurso}. Ca să vedeți cum lucrăm, implementăm fără cost 3 soluții rapide în propria voastră operațiune. Ați fi deschis la o întâlnire ca să vedem dacă are sens să lucrăm împreună? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7703,17 +7703,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho}. You bring in the demand; we work on the layer after the lead: how the request reaches the team, what context travels with it, who decides and how it gets delivered. We don't replace marketing or branding, we protect the result you already generate. I sketched a mini-map for one of your typical clients: {percurso}. Would you be open to a meeting to see whether it makes sense to work together? I'll come prepared.</t>
+          <t>{saudacao} Revin cu un exemplu concret de colaborare: {valor} Voi păstrați relația și serviciul, noi intrăm doar pe partea operațională. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7725,95 +7725,95 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Following up with one concrete collaboration example: {valor} You keep the relationship and the service; we only step into the operational side. I'll come prepared.</t>
+          <t>{saudacao} Mă bucur că cele 3 soluții funcționează deja în echipa voastră. Vă propun un parteneriat simplu. Dacă vi se pare corect, menționați Pacheco Studios ca pe cei care v-au ajutat: o postare cu @pachecostudiospt și un rând pe site. Apoi, când un client de-al vostru se blochează după lead, ne faceți o introducere, cu acordul lui. Voi păstrați clientul și serviciul. Pentru fiecare lucrare care vine din recomandarea voastră primiți 15% din valoarea ei, plătit în 7 zile de la plata clientului. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Punctul despre {tema} mi se pare esențial. În operațiunile pe care le analizez, întrebarea care schimbă cel mai mult este: {pergunta}</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho}. Vocês trazem a procura; nós trabalhamos na camada depois do lead: como o pedido chega à equipa, que contexto leva, quem decide e como se entrega. Não substituímos o marketing nem a marca, protegemos o resultado que vocês já geram. Esbocei um mini-mapa para um cliente típico vosso: {percurso}. Para verem como trabalhamos, implementamos sem custo 3 soluções rápidas na vossa própria operação. Estariam abertos a uma reunião para ver se faz sentido trabalharmos juntos? Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Bună observație. Aș adăuga un detaliu din practică: {valor}</t>
+          <t>{saudacao} Volto com um exemplo concreto de colaboração: {valor} Vocês mantêm a relação e o serviço, nós entramos só na parte operacional. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>O întrebare sinceră pentru cei care au trecut prin asta: {pergunta}</t>
+          <t>{saudacao} Fico contente por as 3 soluções já estarem a funcionar na vossa equipa. Proponho uma parceria simples. Se vos parecer justo, mencionem a Pacheco Studios como quem vos ajudou: um post com @pachecostudiospt e uma linha no site. Depois, quando um cliente vosso encravar depois do lead, apresentam-nos, com o acordo dele. Vocês mantêm o cliente e o serviço. Por cada trabalho que vier da vossa recomendação recebem 15% do valor, pago até 7 dias depois de o cliente pagar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -7823,19 +7823,19 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am comentat în ultimele săptămâni la postările voastre despre {tema}. Lucrez pe sisteme cu AI pentru operațiuni: unde stă contextul, cine răspunde de pasul următor și unde decide un om. Cred că publicul vostru ar găsi util un subiect ca acesta: {gancho}, ca articol, workshop scurt sau discuție la un eveniment. Ați fi deschis la o întâlnire scurtă? Voi fi pregătit.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho}. You bring in the demand; we work on the layer after the lead: how the request reaches the team, what context travels with it, who decides and how it gets delivered. We don't replace marketing or branding, we protect the result you already generate. I sketched a mini-map for one of your typical clients: {percurso}. To show you how we work, we implement 3 quick wins in your own operation at no cost. Would you be open to a meeting to see whether it makes sense to work together? I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -7845,29 +7845,29 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu propunerea de subiect, acum mai concretă: {valor} Mă adaptez formatului care vă ajută cel mai mult. Voi fi pregătit.</t>
+          <t>{saudacao} Following up with one concrete collaboration example: {valor} You keep the relationship and the service; we only step into the operational side. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>O ponto sobre {tema} parece-me essencial. Nas operações que analiso, a pergunta que mais muda o resultado é: {pergunta}</t>
+          <t>{saudacao} Glad the 3 quick wins are already working for your team. I'd like to propose a simple partnership. If it feels fair, mention Pacheco Studios as the team that helped you: a post tagging @pachecostudiospt and a line on your site. Then, when one of your clients gets stuck after the lead, introduce us, with their consent. You keep the client and the service. For every job that comes from your referral you get 15% of its value, paid within 7 days of the client paying. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -7879,17 +7879,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>Comentário: ponto</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Boa observação. Acrescentava um detalhe da prática: {valor}</t>
+          <t>Punctul despre {tema} mi se pare esențial. În operațiunile pe care le analizez, întrebarea care schimbă cel mai mult este: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -7901,17 +7901,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>Comentário: acréscimo</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Uma pergunta sincera para quem já passou por isto: {pergunta}</t>
+          <t>Bună observație. Aș adăuga un detaliu din practică: {valor}</t>
         </is>
       </c>
     </row>
@@ -7923,17 +7923,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Comentário: pergunta</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Tenho comentado nas vossas publicações sobre {tema}. Trabalho em sistemas com IA para operações: onde fica o contexto, quem é dono do próximo passo e onde decide uma pessoa. Acho que a vossa audiência ia achar útil um tema como este: {gancho}, em artigo, workshop curto ou conversa num evento. Estariam abertos a uma reunião curta? Vou estar preparado.</t>
+          <t>O întrebare sinceră pentru cei care au trecut prin asta: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -7945,17 +7945,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto à proposta de tema, agora mais concreta: {valor} Adapto-me ao formato que mais vos ajudar. Vou estar preparado.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am comentat în ultimele săptămâni la postările voastre despre {tema}. Lucrez pe sisteme cu AI pentru operațiuni: unde stă contextul, cine răspunde de pasul următor și unde decide un om. Cred că publicul vostru ar găsi util un subiect ca acesta: {gancho}, ca articol, workshop scurt sau discuție la un eveniment. Ați fi deschis la o întâlnire scurtă? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7967,17 +7967,17 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>The point about {tema} is key. In the operations I map, the question that changes the most is: {pergunta}</t>
+          <t>{saudacao} Revin cu propunerea de subiect, acum mai concretă: {valor} Mă adaptez formatului care vă ajută cel mai mult. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7989,17 +7989,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>Comentário: ponto</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Good point. One detail from practice I'd add: {valor}</t>
+          <t>O ponto sobre {tema} parece-me essencial. Nas operações que analiso, a pergunta que mais muda o resultado é: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -8011,17 +8011,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>Comentário: acréscimo</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>An honest question for anyone who's been through this: {pergunta}</t>
+          <t>Boa observação. Acrescentava um detalhe da prática: {valor}</t>
         </is>
       </c>
     </row>
@@ -8033,17 +8033,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Comentário: pergunta</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I've been commenting on your posts about {tema}. I work on AI systems for operations: where context lives, who owns the next step and where a human decides. I think your audience would find a topic like this useful: {gancho}, as an article, a short workshop or a talk at an event. Would you be open to a short meeting? I'll come prepared.</t>
+          <t>Uma pergunta sincera para quem já passou por isto: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -8055,15 +8055,147 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>DM 1</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Tenho comentado nas vossas publicações sobre {tema}. Trabalho em sistemas com IA para operações: onde fica o contexto, quem é dono do próximo passo e onde decide uma pessoa. Acho que a vossa audiência ia achar útil um tema como este: {gancho}, em artigo, workshop curto ou conversa num evento. Estariam abertos a uma reunião curta? Vou estar preparado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>{saudacao} Volto à proposta de tema, agora mais concreta: {valor} Adapto-me ao formato que mais vos ajudar. Vou estar preparado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
           <t>en</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Comentário: ponto</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>The point about {tema} is key. In the operations I map, the question that changes the most is: {pergunta}</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Comentário: acréscimo</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Good point. One detail from practice I'd add: {valor}</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Comentário: pergunta</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>An honest question for anyone who's been through this: {pergunta}</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>DM 1</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I've been commenting on your posts about {tema}. I work on AI systems for operations: where context lives, who owns the next step and where a human decides. I think your audience would find a topic like this useful: {gancho}, as an article, a short workshop or a talk at an event. Would you be open to a short meeting? I'll come prepared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>{saudacao} Following up on the topic idea, now more concrete: {valor} Happy to fit whatever format helps you most. I'll come prepared.</t>
         </is>

</xml_diff>

<commit_message>
Instagram: 19 DMs de hoje com o ângulo EUA/China, brief de autoridade (RO/PT) e guião para a mesa
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bCka4TNe6PKPBEx4M62DX
</commit_message>
<xml_diff>
--- a/research/instagram/prospecao-instagram.xlsx
+++ b/research/instagram/prospecao-instagram.xlsx
@@ -7361,7 +7361,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho} și m-am gândit la partea din spate a operațiunii tale: {percurso}. Vreau să-ți ofer ceva concret, fără cost: pornind de la situația ta de acum, implementăm 3 soluții rapide în operațiunea ta. Întrebarea de la care pornesc: {pergunta} Ai fi deschis la o scurtă întâlnire ca să alegem împreună cele 3 soluții? Voi fi pregătit.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho} și m-am gândit la partea din spate a operațiunii tale: {percurso}. Companii din SUA și China rezolvă exact asta cu sisteme AI cu reguli clare și cu un om la decizie; în România, doar 5% dintre firme folosesc AI (Eurostat, 2025). Vreau să-ți ofer ceva concret, fără cost: pornind de la situația ta de acum, implementăm 3 soluții rapide în operațiunea ta. Întrebarea de la care pornesc: {pergunta} Ai fi deschis la o scurtă întâlnire ca să alegem împreună cele 3 soluții? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7427,7 +7427,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho} e fiquei a pensar na parte de trás da tua operação: {percurso}. Quero oferecer-te uma coisa concreta, sem custo: a partir da tua situação atual, implementamos 3 soluções rápidas na tua operação. A pergunta de onde parto: {pergunta} Estarias aberto a uma conversa curta para escolhermos juntos as 3 soluções? Vou estar preparado.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho} e fiquei a pensar na parte de trás da tua operação: {percurso}. Empresas dos EUA e da China resolvem exatamente isto com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Quero oferecer-te uma coisa concreta, sem custo: a partir da tua situação atual, implementamos 3 soluções rápidas na tua operação. A pergunta de onde parto: {pergunta} Estarias aberto a uma conversa curta para escolhermos juntos as 3 soluções? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7493,7 +7493,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho} and started thinking about the back end of your operation: {percurso}. I'd like to offer you something concrete, at no cost: based on where your operation is today, we implement 3 quick wins in it. The question I start from: {pergunta} Would you be open to a short call to pick the 3 together? I'll come prepared.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho} and started thinking about the back end of your operation: {percurso}. Companies in the US and China already solve exactly this with AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). I'd like to offer you something concrete, at no cost: based on where your operation is today, we implement 3 quick wins in it. The question I start from: {pergunta} Would you be open to a short call to pick the 3 together? I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -7559,7 +7559,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am parcurs traseul public al unui client {empresa}: {percurso}. Pe baza a ceea ce este public, am o ipoteză de diagnostic, nu o concluzie: {pergunta} Am pus-o pe o mini-hartă de o pagină. Cu cine din echipă ar fi potrivit să o validez: operațiuni, experiența clienților sau transformare digitală? O întâlnire scurtă de explorare ar fi suficientă. Voi fi pregătit.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Companii din SUA și China își conduc deja operațiunile cu sisteme AI cu reguli clare și cu un om la decizie; în România, doar 5% dintre firme folosesc AI (Eurostat, 2025). Am parcurs traseul public al unui client {empresa}: {percurso}. Pe baza a ceea ce este public, am o ipoteză de diagnostic, nu o concluzie: {pergunta} Am pus-o pe o mini-hartă de o pagină și pot implementa fără cost 3 soluții rapide ca să o testăm. Cu cine din echipă ar fi potrivit să o validez: operațiuni, experiența clienților sau transformare digitală? O întâlnire scurtă de explorare ar fi suficientă. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7603,7 +7603,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Percorri o percurso público de um cliente {empresa}: {percurso}. Com base no que é público, tenho uma hipótese de diagnóstico, não uma conclusão: {pergunta} Pus isto num mini-mapa de uma página. Quem na equipa seria a pessoa certa para o validar: operações, experiência do cliente ou transformação digital? Uma conversa exploratória curta chega. Vou estar preparado.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Empresas dos EUA e da China já conduzem as operações com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Percorri o percurso público de um cliente {empresa}: {percurso}. Com base no que é público, tenho uma hipótese de diagnóstico, não uma conclusão: {pergunta} Pus isto num mini-mapa de uma página e posso implementar sem custo 3 soluções rápidas para a testarmos. Quem na equipa seria a pessoa certa para o validar: operações, experiência do cliente ou transformação digital? Uma conversa exploratória curta chega. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7647,7 +7647,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I walked through the public journey of a {empresa} customer: {percurso}. Based only on what's public, I have a diagnostic hypothesis, not a conclusion: {pergunta} I've put it on a one-page mini-map. Who on the team would be the right person to validate it: operations, customer experience or digital transformation? A short exploratory call would be enough. I'll come prepared.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. Companies in the US and China already run their operations on AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). I walked through the public journey of a {empresa} customer: {percurso}. Based only on what's public, I have a diagnostic hypothesis, not a conclusion: {pergunta} I've put it on a one-page mini-map and can implement 3 quick wins at no cost so we can test it. Who on the team would be the right person to validate it: operations, customer experience or digital transformation? A short exploratory call would be enough. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -7691,7 +7691,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho}. Voi aduceți cererea; noi lucrăm în stratul de după lead: cum ajunge cererea la echipă, ce context o însoțește, cine decide și cum se livrează. Nu înlocuim marketingul sau brandingul, protejăm rezultatul pe care îl generați deja. Am schițat o mini-hartă pentru un client tipic de-al vostru: {percurso}. Ca să vedeți cum lucrăm, implementăm fără cost 3 soluții rapide în propria voastră operațiune. Ați fi deschis la o întâlnire ca să vedem dacă are sens să lucrăm împreună? Voi fi pregătit.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho}. Companii din SUA și China își conduc deja operațiunile cu sisteme AI cu reguli clare și cu un om la decizie; în România, doar 5% dintre firme folosesc AI (Eurostat, 2025). Voi aduceți cererea; noi lucrăm în stratul de după lead: cum ajunge cererea la echipă, ce context o însoțește, cine decide și cum se livrează. Nu înlocuim marketingul sau brandingul, protejăm rezultatul pe care îl generați deja. Am schițat o mini-hartă pentru un client tipic de-al vostru: {percurso}. Ca să vedeți cum lucrăm, implementăm fără cost 3 soluții rapide în propria voastră operațiune. Ați fi deschis la o întâlnire ca să vedem dacă are sens să lucrăm împreună? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7757,7 +7757,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho}. Vocês trazem a procura; nós trabalhamos na camada depois do lead: como o pedido chega à equipa, que contexto leva, quem decide e como se entrega. Não substituímos o marketing nem a marca, protegemos o resultado que vocês já geram. Esbocei um mini-mapa para um cliente típico vosso: {percurso}. Para verem como trabalhamos, implementamos sem custo 3 soluções rápidas na vossa própria operação. Estariam abertos a uma reunião para ver se faz sentido trabalharmos juntos? Vou estar preparado.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho}. Empresas dos EUA e da China já conduzem as operações com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Vocês trazem a procura; nós trabalhamos na camada depois do lead: como o pedido chega à equipa, que contexto leva, quem decide e como se entrega. Não substituímos o marketing nem a marca, protegemos o resultado que vocês já geram. Esbocei um mini-mapa para um cliente típico vosso: {percurso}. Para verem como trabalhamos, implementamos sem custo 3 soluções rápidas na vossa própria operação. Estariam abertos a uma reunião para ver se faz sentido trabalharmos juntos? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7823,7 +7823,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho}. You bring in the demand; we work on the layer after the lead: how the request reaches the team, what context travels with it, who decides and how it gets delivered. We don't replace marketing or branding, we protect the result you already generate. I sketched a mini-map for one of your typical clients: {percurso}. To show you how we work, we implement 3 quick wins in your own operation at no cost. Would you be open to a meeting to see whether it makes sense to work together? I'll come prepared.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho}. Companies in the US and China already run their operations on AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). You bring in the demand; we work on the layer after the lead: how the request reaches the team, what context travels with it, who decides and how it gets delivered. We don't replace marketing or branding, we protect the result you already generate. I sketched a mini-map for one of your typical clients: {percurso}. To show you how we work, we implement 3 quick wins in your own operation at no cost. Would you be open to a meeting to see whether it makes sense to work together? I'll come prepared.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Instagram alinhado com o playbook de consultoria: escada quick wins → triagem → auditoria, CTA DM AUDIT, comissão suspensa
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bCka4TNe6PKPBEx4M62DX
</commit_message>
<xml_diff>
--- a/research/instagram/prospecao-instagram.xlsx
+++ b/research/instagram/prospecao-instagram.xlsx
@@ -730,7 +730,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Conversa → 3 quick wins implementados → mostram o nosso nome por gratidão → recomendam, com 15% de cada trabalho que vier deles.</t>
+          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
@@ -838,7 +838,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Conversa → 3 quick wins implementados → mostram o nosso nome por gratidão → recomendam, com 15% de cada trabalho que vier deles.</t>
+          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="O3" s="2" t="n">
@@ -946,7 +946,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Conversa → 3 quick wins implementados → mostram o nosso nome por gratidão → recomendam, com 15% de cada trabalho que vier deles.</t>
+          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="O4" s="2" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Conversa → 3 quick wins implementados → mostram o nosso nome por gratidão → recomendam, com 15% de cada trabalho que vier deles.</t>
+          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="O5" s="2" t="n">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Encaminhamento para o dono do processo ou reunião de descoberta que converta numa AI Systems Audit.</t>
+          <t>Encaminhamento para o dono do processo → triagem curta → Auditoria de Sistemas com IA → sprint de desenho → piloto controlado.</t>
         </is>
       </c>
       <c r="O6" s="2" t="n">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="O7" s="2" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="O8" s="2" t="n">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="O9" s="2" t="n">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="O10" s="2" t="n">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="O11" s="2" t="n">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="O12" s="2" t="n">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo, evento ou referência.</t>
+          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo de diagnóstico, evento ou pedidos AUDIT.</t>
         </is>
       </c>
       <c r="O13" s="2" t="n">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo, evento ou referência.</t>
+          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo de diagnóstico, evento ou pedidos AUDIT.</t>
         </is>
       </c>
       <c r="O14" s="2" t="n">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo, evento ou referência.</t>
+          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo de diagnóstico, evento ou pedidos AUDIT.</t>
         </is>
       </c>
       <c r="O15" s="2" t="n">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo, evento ou referência.</t>
+          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo de diagnóstico, evento ou pedidos AUDIT.</t>
         </is>
       </c>
       <c r="O16" s="2" t="n">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo, evento ou referência.</t>
+          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo de diagnóstico, evento ou pedidos AUDIT.</t>
         </is>
       </c>
       <c r="O17" s="2" t="n">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo, evento ou referência.</t>
+          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo de diagnóstico, evento ou pedidos AUDIT.</t>
         </is>
       </c>
       <c r="O18" s="2" t="n">
@@ -7161,7 +7161,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Parceria de prova e indicações qualificadas.</t>
+          <t>Prova com 3 quick wins; depois triagem e auditoria; indicações qualificadas.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -7181,7 +7181,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Conversa → 3 quick wins implementados → mostram o nosso nome por gratidão → recomendam, com 15% de cada trabalho que vier deles.</t>
+          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Encaminhamento para o dono do processo ou reunião de descoberta que converta numa AI Systems Audit.</t>
+          <t>Encaminhamento para o dono do processo → triagem curta → Auditoria de Sistemas com IA → sprint de desenho → piloto controlado.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -7255,7 +7255,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → mostram o nosso nome → recomendam clientes, com 15% de cada trabalho que vier deles; co-entrega quando fizer sentido.</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -7292,7 +7292,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo, evento ou referência.</t>
+          <t>Familiaridade perante a audiência → DM ou introdução → conteúdo de diagnóstico, evento ou pedidos AUDIT.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7400,12 +7400,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Mă bucur că cele 3 soluții merg deja la tine. Am o propunere simplă de parteneriat. Dacă ți se pare corect, menționează Pacheco Studios ca pe cei care te-au ajutat: o postare sau un story cu @pachecostudiospt și un rând pe site. Apoi, când întâlnești o afacere care se blochează în același loc, ne faci o introducere, cu acordul ei. Pentru fiecare lucrare care vine din recomandarea ta primești 15% din valoarea ei, plătit în 7 zile de la plata clientului. Voi fi pregătit.</t>
+          <t>{saudacao} Mulțumesc pentru răspuns. Ca să nu vă ocup timpul, trei întrebări scurte de triaj: ce rezultat operațional vreți să îmbunătățiți în următoarele 90 de zile; unde intră azi cererea și unde se blochează sau cere pe cineva să alerge după ea; cine e responsabil de pasul următor. Cu răspunsurile pregătesc harta și cele 3 soluții rapide. Apoi decidem împreună dacă are sens un Audit de Sisteme cu AI. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7466,12 +7466,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Fico contente por as 3 soluções já estarem a funcionar contigo. Tenho uma proposta simples de parceria. Se te parecer justo, menciona a Pacheco Studios como quem te ajudou: um post ou story com @pachecostudiospt e uma linha no site. Depois, quando conheceres um negócio que encrava no mesmo sítio, apresentas-nos, com o acordo dele. Por cada trabalho que vier da tua recomendação recebes 15% do valor, pago até 7 dias depois de o cliente pagar. Vou estar preparado.</t>
+          <t>{saudacao} Obrigado pela resposta. Para não vos ocupar tempo, três perguntas curtas de triagem: que resultado operacional querem melhorar nos próximos 90 dias; onde entra hoje o pedido e onde abranda ou obriga alguém a correr atrás dele; quem é dono do próximo passo. Com as respostas preparo o mapa e as 3 soluções rápidas. Depois decidimos juntos se faz sentido uma Auditoria de Sistemas com IA. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7532,12 +7532,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Glad the 3 quick wins are already working for you. I have a simple partnership proposal. If it feels fair, mention Pacheco Studios as the team that helped you: a post or story tagging @pachecostudiospt and a line on your site. Then, when you meet a business stuck in the same place, introduce us, with their consent. For every job that comes from your referral you get 15% of its value, paid within 7 days of the client paying. I'll come prepared.</t>
+          <t>{saudacao} Thanks for getting back to me. To keep it short, three triage questions: which operational result do you want to improve in the next 90 days; where does a request come in today and where does it slow down or need someone chasing it; who owns the next step. With your answers I prepare the map and the 3 quick wins. Then we decide together whether an AI Systems Audit makes sense. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -7593,17 +7593,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Empresas dos EUA e da China já conduzem as operações com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Percorri o percurso público de um cliente {empresa}: {percurso}. Com base no que é público, tenho uma hipótese de diagnóstico, não uma conclusão: {pergunta} Pus isto num mini-mapa de uma página e posso implementar sem custo 3 soluções rápidas para a testarmos. Quem na equipa seria a pessoa certa para o validar: operações, experiência do cliente ou transformação digital? Uma conversa exploratória curta chega. Vou estar preparado.</t>
+          <t>{saudacao} Mulțumesc pentru răspuns. Ca să nu vă ocup timpul, trei întrebări scurte de triaj: ce rezultat operațional vreți să îmbunătățiți în următoarele 90 de zile; unde intră azi cererea și unde se blochează sau cere pe cineva să alerge după ea; cine e responsabil de pasul următor. Cu răspunsurile pregătesc harta și cele 3 soluții rapide. Apoi decidem împreună dacă are sens un Audit de Sisteme cu AI. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7620,12 +7620,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto ao mini-mapa sobre o percurso do cliente {empresa}. Acrescentei um único ponto: {valor} Se me puderem indicar a pessoa certa, envio-lhe o mapa diretamente. Vou estar preparado.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Empresas dos EUA e da China já conduzem as operações com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Percorri o percurso público de um cliente {empresa}: {percurso}. Com base no que é público, tenho uma hipótese de diagnóstico, não uma conclusão: {pergunta} Pus isto num mini-mapa de uma página e posso implementar sem custo 3 soluções rápidas para a testarmos. Quem na equipa seria a pessoa certa para o validar: operações, experiência do cliente ou transformação digital? Uma conversa exploratória curta chega. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7637,17 +7637,17 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. Companies in the US and China already run their operations on AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). I walked through the public journey of a {empresa} customer: {percurso}. Based only on what's public, I have a diagnostic hypothesis, not a conclusion: {pergunta} I've put it on a one-page mini-map and can implement 3 quick wins at no cost so we can test it. Who on the team would be the right person to validate it: operations, customer experience or digital transformation? A short exploratory call would be enough. I'll come prepared.</t>
+          <t>{saudacao} Volto ao mini-mapa sobre o percurso do cliente {empresa}. Acrescentei um único ponto: {valor} Se me puderem indicar a pessoa certa, envio-lhe o mapa diretamente. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7659,29 +7659,29 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Following up on the mini-map of the {empresa} customer journey. I added one point: {valor} If you can point me to the right person, I'll send the map to them directly. I'll come prepared.</t>
+          <t>{saudacao} Obrigado pela resposta. Para não vos ocupar tempo, três perguntas curtas de triagem: que resultado operacional querem melhorar nos próximos 90 dias; onde entra hoje o pedido e onde abranda ou obriga alguém a correr atrás dele; quem é dono do próximo passo. Com as respostas preparo o mapa e as 3 soluções rápidas. Depois decidimos juntos se faz sentido uma Auditoria de Sistemas com IA. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -7691,19 +7691,19 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho}. Companii din SUA și China își conduc deja operațiunile cu sisteme AI cu reguli clare și cu un om la decizie; în România, doar 5% dintre firme folosesc AI (Eurostat, 2025). Voi aduceți cererea; noi lucrăm în stratul de după lead: cum ajunge cererea la echipă, ce context o însoțește, cine decide și cum se livrează. Nu înlocuim marketingul sau brandingul, protejăm rezultatul pe care îl generați deja. Am schițat o mini-hartă pentru un client tipic de-al vostru: {percurso}. Ca să vedeți cum lucrăm, implementăm fără cost 3 soluții rapide în propria voastră operațiune. Ați fi deschis la o întâlnire ca să vedem dacă are sens să lucrăm împreună? Voi fi pregătit.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. Companies in the US and China already run their operations on AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). I walked through the public journey of a {empresa} customer: {percurso}. Based only on what's public, I have a diagnostic hypothesis, not a conclusion: {pergunta} I've put it on a one-page mini-map and can implement 3 quick wins at no cost so we can test it. Who on the team would be the right person to validate it: operations, customer experience or digital transformation? A short exploratory call would be enough. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -7713,29 +7713,29 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu un exemplu concret de colaborare: {valor} Voi păstrați relația și serviciul, noi intrăm doar pe partea operațională. Voi fi pregătit.</t>
+          <t>{saudacao} Following up on the mini-map of the {empresa} customer journey. I added one point: {valor} If you can point me to the right person, I'll send the map to them directly. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Mă bucur că cele 3 soluții funcționează deja în echipa voastră. Vă propun un parteneriat simplu. Dacă vi se pare corect, menționați Pacheco Studios ca pe cei care v-au ajutat: o postare cu @pachecostudiospt și un rând pe site. Apoi, când un client de-al vostru se blochează după lead, ne faceți o introducere, cu acordul lui. Voi păstrați clientul și serviciul. Pentru fiecare lucrare care vine din recomandarea voastră primiți 15% din valoarea ei, plătit în 7 zile de la plata clientului. Voi fi pregătit.</t>
+          <t>{saudacao} Thanks for getting back to me. To keep it short, three triage questions: which operational result do you want to improve in the next 90 days; where does a request come in today and where does it slow down or need someone chasing it; who owns the next step. With your answers I prepare the map and the 3 quick wins. Then we decide together whether an AI Systems Audit makes sense. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -7747,7 +7747,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho}. Empresas dos EUA e da China já conduzem as operações com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Vocês trazem a procura; nós trabalhamos na camada depois do lead: como o pedido chega à equipa, que contexto leva, quem decide e como se entrega. Não substituímos o marketing nem a marca, protegemos o resultado que vocês já geram. Esbocei um mini-mapa para um cliente típico vosso: {percurso}. Para verem como trabalhamos, implementamos sem custo 3 soluções rápidas na vossa própria operação. Estariam abertos a uma reunião para ver se faz sentido trabalharmos juntos? Vou estar preparado.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho}. Companii din SUA și China își conduc deja operațiunile cu sisteme AI cu reguli clare și cu un om la decizie; în România, doar 5% dintre firme folosesc AI (Eurostat, 2025). Voi aduceți cererea; noi lucrăm în stratul de după lead: cum ajunge cererea la echipă, ce context o însoțește, cine decide și cum se livrează. Nu înlocuim marketingul sau brandingul, protejăm rezultatul pe care îl generați deja. Am schițat o mini-hartă pentru un client tipic de-al vostru: {percurso}. Ca să vedeți cum lucrăm, implementăm fără cost 3 soluții rapide în propria voastră operațiune. Ați fi deschis la o întâlnire ca să vedem dacă are sens să lucrăm împreună? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7769,7 +7769,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto com um exemplo concreto de colaboração: {valor} Vocês mantêm a relação e o serviço, nós entramos só na parte operacional. Vou estar preparado.</t>
+          <t>{saudacao} Revin cu un exemplu concret de colaborare: {valor} Voi păstrați relația și serviciul, noi intrăm doar pe partea operațională. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7791,17 +7791,17 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Fico contente por as 3 soluções já estarem a funcionar na vossa equipa. Proponho uma parceria simples. Se vos parecer justo, mencionem a Pacheco Studios como quem vos ajudou: um post com @pachecostudiospt e uma linha no site. Depois, quando um cliente vosso encravar depois do lead, apresentam-nos, com o acordo dele. Vocês mantêm o cliente e o serviço. Por cada trabalho que vier da vossa recomendação recebem 15% do valor, pago até 7 dias depois de o cliente pagar. Vou estar preparado.</t>
+          <t>{saudacao} Mulțumesc pentru răspuns. Ca să nu vă ocup timpul, trei întrebări scurte de triaj: ce rezultat operațional vreți să îmbunătățiți în următoarele 90 de zile; unde intră azi cererea și unde se blochează sau cere pe cineva să alerge după ea; cine e responsabil de pasul următor. Cu răspunsurile pregătesc harta și cele 3 soluții rapide. Apoi decidem împreună dacă are sens un Audit de Sisteme cu AI. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7813,7 +7813,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho}. Companies in the US and China already run their operations on AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). You bring in the demand; we work on the layer after the lead: how the request reaches the team, what context travels with it, who decides and how it gets delivered. We don't replace marketing or branding, we protect the result you already generate. I sketched a mini-map for one of your typical clients: {percurso}. To show you how we work, we implement 3 quick wins in your own operation at no cost. Would you be open to a meeting to see whether it makes sense to work together? I'll come prepared.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho}. Empresas dos EUA e da China já conduzem as operações com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Vocês trazem a procura; nós trabalhamos na camada depois do lead: como o pedido chega à equipa, que contexto leva, quem decide e como se entrega. Não substituímos o marketing nem a marca, protegemos o resultado que vocês já geram. Esbocei um mini-mapa para um cliente típico vosso: {percurso}. Para verem como trabalhamos, implementamos sem custo 3 soluções rápidas na vossa própria operação. Estariam abertos a uma reunião para ver se faz sentido trabalharmos juntos? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7835,7 +7835,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -7845,7 +7845,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Following up with one concrete collaboration example: {valor} You keep the relationship and the service; we only step into the operational side. I'll come prepared.</t>
+          <t>{saudacao} Volto com um exemplo concreto de colaboração: {valor} Vocês mantêm a relação e o serviço, nós entramos só na parte operacional. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7857,83 +7857,83 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Glad the 3 quick wins are already working for your team. I'd like to propose a simple partnership. If it feels fair, mention Pacheco Studios as the team that helped you: a post tagging @pachecostudiospt and a line on your site. Then, when one of your clients gets stuck after the lead, introduce us, with their consent. You keep the client and the service. For every job that comes from your referral you get 15% of its value, paid within 7 days of the client paying. I'll come prepared.</t>
+          <t>{saudacao} Obrigado pela resposta. Para não vos ocupar tempo, três perguntas curtas de triagem: que resultado operacional querem melhorar nos próximos 90 dias; onde entra hoje o pedido e onde abranda ou obriga alguém a correr atrás dele; quem é dono do próximo passo. Com as respostas preparo o mapa e as 3 soluções rápidas. Depois decidimos juntos se faz sentido uma Auditoria de Sistemas com IA. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Punctul despre {tema} mi se pare esențial. În operațiunile pe care le analizez, întrebarea care schimbă cel mai mult este: {pergunta}</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho}. Companies in the US and China already run their operations on AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). You bring in the demand; we work on the layer after the lead: how the request reaches the team, what context travels with it, who decides and how it gets delivered. We don't replace marketing or branding, we protect the result you already generate. I sketched a mini-map for one of your typical clients: {percurso}. To show you how we work, we implement 3 quick wins in your own operation at no cost. Would you be open to a meeting to see whether it makes sense to work together? I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Bună observație. Aș adăuga un detaliu din practică: {valor}</t>
+          <t>{saudacao} Following up with one concrete collaboration example: {valor} You keep the relationship and the service; we only step into the operational side. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>O întrebare sinceră pentru cei care au trecut prin asta: {pergunta}</t>
+          <t>{saudacao} Thanks for getting back to me. To keep it short, three triage questions: which operational result do you want to improve in the next 90 days; where does a request come in today and where does it slow down or need someone chasing it; who owns the next step. With your answers I prepare the map and the 3 quick wins. Then we decide together whether an AI Systems Audit makes sense. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -7950,12 +7950,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Comentário: ponto</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am comentat în ultimele săptămâni la postările voastre despre {tema}. Lucrez pe sisteme cu AI pentru operațiuni: unde stă contextul, cine răspunde de pasul următor și unde decide un om. Cred că publicul vostru ar găsi util un subiect ca acesta: {gancho}, ca articol, workshop scurt sau discuție la un eveniment. Ați fi deschis la o întâlnire scurtă? Voi fi pregătit.</t>
+          <t>Punctul despre {tema} mi se pare esențial. În operațiunile pe care le analizez, întrebarea care schimbă cel mai mult este: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -7972,12 +7972,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Comentário: acréscimo</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu propunerea de subiect, acum mai concretă: {valor} Mă adaptez formatului care vă ajută cel mai mult. Voi fi pregătit.</t>
+          <t>Bună observație. Aș adăuga un detaliu din practică: {valor}</t>
         </is>
       </c>
     </row>
@@ -7989,17 +7989,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>Comentário: pergunta</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>O ponto sobre {tema} parece-me essencial. Nas operações que analiso, a pergunta que mais muda o resultado é: {pergunta}</t>
+          <t>O întrebare sinceră pentru cei care au trecut prin asta: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -8011,17 +8011,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Boa observação. Acrescentava um detalhe da prática: {valor}</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am comentat în ultimele săptămâni la postările voastre despre {tema}. Lucrez pe sisteme cu AI pentru operațiuni: unde stă contextul, cine răspunde de pasul următor și unde decide un om. Cred că publicul vostru ar găsi util un subiect ca acesta: {gancho}, ca articol, workshop scurt sau discuție la un eveniment. Ați fi deschis la o întâlnire scurtă? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -8033,17 +8033,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Uma pergunta sincera para quem já passou por isto: {pergunta}</t>
+          <t>{saudacao} Revin cu propunerea de subiect, acum mai concretă: {valor} Mă adaptez formatului care vă ajută cel mai mult. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -8060,12 +8060,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Comentário: ponto</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Tenho comentado nas vossas publicações sobre {tema}. Trabalho em sistemas com IA para operações: onde fica o contexto, quem é dono do próximo passo e onde decide uma pessoa. Acho que a vossa audiência ia achar útil um tema como este: {gancho}, em artigo, workshop curto ou conversa num evento. Estariam abertos a uma reunião curta? Vou estar preparado.</t>
+          <t>O ponto sobre {tema} parece-me essencial. Nas operações que analiso, a pergunta que mais muda o resultado é: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -8082,12 +8082,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Comentário: acréscimo</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto à proposta de tema, agora mais concreta: {valor} Adapto-me ao formato que mais vos ajudar. Vou estar preparado.</t>
+          <t>Boa observação. Acrescentava um detalhe da prática: {valor}</t>
         </is>
       </c>
     </row>
@@ -8099,17 +8099,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>Comentário: pergunta</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>The point about {tema} is key. In the operations I map, the question that changes the most is: {pergunta}</t>
+          <t>Uma pergunta sincera para quem já passou por isto: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -8121,17 +8121,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Good point. One detail from practice I'd add: {valor}</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Tenho comentado nas vossas publicações sobre {tema}. Trabalho em sistemas com IA para operações: onde fica o contexto, quem é dono do próximo passo e onde decide uma pessoa. Acho que a vossa audiência ia achar útil um tema como este: {gancho}, em artigo, workshop curto ou conversa num evento. Estariam abertos a uma reunião curta? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -8143,17 +8143,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>An honest question for anyone who's been through this: {pergunta}</t>
+          <t>{saudacao} Volto à proposta de tema, agora mais concreta: {valor} Adapto-me ao formato que mais vos ajudar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -8170,12 +8170,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Comentário: ponto</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I've been commenting on your posts about {tema}. I work on AI systems for operations: where context lives, who owns the next step and where a human decides. I think your audience would find a topic like this useful: {gancho}, as an article, a short workshop or a talk at an event. Would you be open to a short meeting? I'll come prepared.</t>
+          <t>The point about {tema} is key. In the operations I map, the question that changes the most is: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -8192,10 +8192,76 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
+          <t>Comentário: acréscimo</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Good point. One detail from practice I'd add: {valor}</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Comentário: pergunta</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>An honest question for anyone who's been through this: {pergunta}</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>DM 1</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I've been commenting on your posts about {tema}. I work on AI systems for operations: where context lives, who owns the next step and where a human decides. I think your audience would find a topic like this useful: {gancho}, as an article, a short workshop or a talk at an event. Would you be open to a short meeting? I'll come prepared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>{saudacao} Following up on the topic idea, now more concrete: {valor} Happy to fit whatever format helps you most. I'll come prepared.</t>
         </is>

</xml_diff>

<commit_message>
Parceiros: 10% a cada 3 meses sobre a implementação; auditoria creditada na implementação; mensagem Parceria de volta
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bCka4TNe6PKPBEx4M62DX
</commit_message>
<xml_diff>
--- a/research/instagram/prospecao-instagram.xlsx
+++ b/research/instagram/prospecao-instagram.xlsx
@@ -730,7 +730,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois (comissão a decidir pelo Tomás).</t>
+          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois: 10% do que faturamos ao negócio indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
@@ -838,7 +838,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois (comissão a decidir pelo Tomás).</t>
+          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois: 10% do que faturamos ao negócio indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="O3" s="2" t="n">
@@ -946,7 +946,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois (comissão a decidir pelo Tomás).</t>
+          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois: 10% do que faturamos ao negócio indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="O4" s="2" t="n">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois (comissão a decidir pelo Tomás).</t>
+          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois: 10% do que faturamos ao negócio indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="O5" s="2" t="n">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 10% do que faturamos ao cliente indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="O7" s="2" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 10% do que faturamos ao cliente indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="O8" s="2" t="n">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 10% do que faturamos ao cliente indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="O9" s="2" t="n">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 10% do que faturamos ao cliente indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="O10" s="2" t="n">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 10% do que faturamos ao cliente indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="O11" s="2" t="n">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 10% do que faturamos ao cliente indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="O12" s="2" t="n">
@@ -7181,7 +7181,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois (comissão a decidir pelo Tomás).</t>
+          <t>Conversa → 3 quick wins → triagem curta → Auditoria de Sistemas com IA; indicações consentidas depois: 10% do que faturamos ao negócio indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -7255,7 +7255,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois (comissão a decidir pelo Tomás).</t>
+          <t>3 quick wins → triagem → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 10% do que faturamos ao cliente indicado, de 3 em 3 meses, enquanto durar.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7417,17 +7417,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho} e fiquei a pensar na parte de trás da tua operação: {percurso}. Empresas dos EUA e da China resolvem exatamente isto com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Quero oferecer-te uma coisa concreta, sem custo: a partir da tua situação atual, implementamos 3 soluções rápidas na tua operação. A pergunta de onde parto: {pergunta} Estarias aberto a uma conversa curta para escolhermos juntos as 3 soluções? Vou estar preparado.</t>
+          <t>{saudacao} Mă bucur că cele 3 soluții merg deja la tine. Am o propunere simplă de parteneriat. Dacă ți se pare corect, menționează Pacheco Studios ca pe cei care te-au ajutat: o postare sau un story cu @pachecostudiospt și un rând pe site. Apoi, când întâlnești o afacere care se blochează în același loc, ne faci o introducere, cu acordul ei. Dacă ajungem să lucrăm cu acea afacere, primești 10% din ce facturăm acolo, plătit la fiecare 3 luni, cât timp colaborarea continuă. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7444,12 +7444,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto só com uma coisa concreta: {valor} A oferta das 3 soluções mantém-se, sem compromisso. Se agora não é o momento, percebo perfeitamente. Vou estar preparado.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho} e fiquei a pensar na parte de trás da tua operação: {percurso}. Empresas dos EUA e da China resolvem exatamente isto com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Quero oferecer-te uma coisa concreta, sem custo: a partir da tua situação atual, implementamos 3 soluções rápidas na tua operação. A pergunta de onde parto: {pergunta} Estarias aberto a uma conversa curta para escolhermos juntos as 3 soluções? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7466,12 +7466,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Triagem (depois da resposta)</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Obrigado pela resposta. Para não vos ocupar tempo, três perguntas curtas de triagem: que resultado operacional querem melhorar nos próximos 90 dias; onde entra hoje o pedido e onde abranda ou obriga alguém a correr atrás dele; quem é dono do próximo passo. Com as respostas preparo o mapa e as 3 soluções rápidas. Depois decidimos juntos se faz sentido uma Auditoria de Sistemas com IA. Vou estar preparado.</t>
+          <t>{saudacao} Volto só com uma coisa concreta: {valor} A oferta das 3 soluções mantém-se, sem compromisso. Se agora não é o momento, percebo perfeitamente. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7483,17 +7483,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho} and started thinking about the back end of your operation: {percurso}. Companies in the US and China already solve exactly this with AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). I'd like to offer you something concrete, at no cost: based on where your operation is today, we implement 3 quick wins in it. The question I start from: {pergunta} Would you be open to a short call to pick the 3 together? I'll come prepared.</t>
+          <t>{saudacao} Obrigado pela resposta. Para não vos ocupar tempo, três perguntas curtas de triagem: que resultado operacional querem melhorar nos próximos 90 dias; onde entra hoje o pedido e onde abranda ou obriga alguém a correr atrás dele; quem é dono do próximo passo. Com as respostas preparo o mapa e as 3 soluções rápidas. Depois decidimos juntos se faz sentido uma Auditoria de Sistemas com IA. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7505,17 +7505,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} A quick follow-up with one concrete thing: {valor} The offer of the 3 quick wins still stands, no strings attached. If now isn't the right time, completely understood. I'll come prepared.</t>
+          <t>{saudacao} Fico contente por as 3 soluções já estarem a funcionar contigo. Tenho uma proposta simples de parceria. Se te parecer justo, menciona a Pacheco Studios como quem te ajudou: um post ou story com @pachecostudiospt e uma linha no site. Depois, quando conheceres um negócio que encrava no mesmo sítio, apresentas-nos, com o acordo dele. Se chegarmos a trabalhar com esse negócio, recebes 10% do que faturamos lá, pago de 3 em 3 meses, enquanto a colaboração durar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7532,78 +7532,78 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Triagem (depois da resposta)</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Thanks for getting back to me. To keep it short, three triage questions: which operational result do you want to improve in the next 90 days; where does a request come in today and where does it slow down or need someone chasing it; who owns the next step. With your answers I prepare the map and the 3 quick wins. Then we decide together whether an AI Systems Audit makes sense. I'll come prepared.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho} and started thinking about the back end of your operation: {percurso}. Companies in the US and China already solve exactly this with AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). I'd like to offer you something concrete, at no cost: based on where your operation is today, we implement 3 quick wins in it. The question I start from: {pergunta} Would you be open to a short call to pick the 3 together? I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Grande negócio</t>
+          <t>Influenciador / operador</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Companii din SUA și China își conduc deja operațiunile cu sisteme AI cu reguli clare și cu un om la decizie; în România, doar 5% dintre firme folosesc AI (Eurostat, 2025). Am parcurs traseul public al unui client {empresa}: {percurso}. Pe baza a ceea ce este public, am o ipoteză de diagnostic, nu o concluzie: {pergunta} Am pus-o pe o mini-hartă de o pagină și pot implementa fără cost 3 soluții rapide ca să o testăm. Cu cine din echipă ar fi potrivit să o validez: operațiuni, experiența clienților sau transformare digitală? O întâlnire scurtă de explorare ar fi suficientă. Voi fi pregătit.</t>
+          <t>{saudacao} A quick follow-up with one concrete thing: {valor} The offer of the 3 quick wins still stands, no strings attached. If now isn't the right time, completely understood. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Grande negócio</t>
+          <t>Influenciador / operador</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu mini-harta despre traseul clientului {empresa}. Am adăugat un singur punct: {valor} Dacă îmi puteți indica persoana potrivită, îi trimit direct harta. Voi fi pregătit.</t>
+          <t>{saudacao} Thanks for getting back to me. To keep it short, three triage questions: which operational result do you want to improve in the next 90 days; where does a request come in today and where does it slow down or need someone chasing it; who owns the next step. With your answers I prepare the map and the 3 quick wins. Then we decide together whether an AI Systems Audit makes sense. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Grande negócio</t>
+          <t>Influenciador / operador</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Triagem (depois da resposta)</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Mulțumesc pentru răspuns. Ca să nu vă ocup timpul, trei întrebări scurte de triaj: ce rezultat operațional vreți să îmbunătățiți în următoarele 90 de zile; unde intră azi cererea și unde se blochează sau cere pe cineva să alerge după ea; cine e responsabil de pasul următor. Cu răspunsurile pregătesc harta și cele 3 soluții rapide. Apoi decidem împreună dacă are sens un Audit de Sisteme cu AI. Voi fi pregătit.</t>
+          <t>{saudacao} Glad the 3 quick wins are already working for you. I have a simple partnership proposal. If it feels fair, mention Pacheco Studios as the team that helped you: a post or story tagging @pachecostudiospt and a line on your site. Then, when you meet a business stuck in the same place, introduce us, with their consent. If we end up working with that business, you get 10% of what we bill there, paid every 3 months for as long as the collaboration lasts. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -7615,7 +7615,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Empresas dos EUA e da China já conduzem as operações com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Percorri o percurso público de um cliente {empresa}: {percurso}. Com base no que é público, tenho uma hipótese de diagnóstico, não uma conclusão: {pergunta} Pus isto num mini-mapa de uma página e posso implementar sem custo 3 soluções rápidas para a testarmos. Quem na equipa seria a pessoa certa para o validar: operações, experiência do cliente ou transformação digital? Uma conversa exploratória curta chega. Vou estar preparado.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Companii din SUA și China își conduc deja operațiunile cu sisteme AI cu reguli clare și cu un om la decizie; în România, doar 5% dintre firme folosesc AI (Eurostat, 2025). Am parcurs traseul public al unui client {empresa}: {percurso}. Pe baza a ceea ce este public, am o ipoteză de diagnostic, nu o concluzie: {pergunta} Am pus-o pe o mini-hartă de o pagină și pot implementa fără cost 3 soluții rapide ca să o testăm. Cu cine din echipă ar fi potrivit să o validez: operațiuni, experiența clienților sau transformare digitală? O întâlnire scurtă de explorare ar fi suficientă. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7637,7 +7637,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto ao mini-mapa sobre o percurso do cliente {empresa}. Acrescentei um único ponto: {valor} Se me puderem indicar a pessoa certa, envio-lhe o mapa diretamente. Vou estar preparado.</t>
+          <t>{saudacao} Revin cu mini-harta despre traseul clientului {empresa}. Am adăugat un singur punct: {valor} Dacă îmi puteți indica persoana potrivită, îi trimit direct harta. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7659,7 +7659,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -7669,7 +7669,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Obrigado pela resposta. Para não vos ocupar tempo, três perguntas curtas de triagem: que resultado operacional querem melhorar nos próximos 90 dias; onde entra hoje o pedido e onde abranda ou obriga alguém a correr atrás dele; quem é dono do próximo passo. Com as respostas preparo o mapa e as 3 soluções rápidas. Depois decidimos juntos se faz sentido uma Auditoria de Sistemas com IA. Vou estar preparado.</t>
+          <t>{saudacao} Mulțumesc pentru răspuns. Ca să nu vă ocup timpul, trei întrebări scurte de triaj: ce rezultat operațional vreți să îmbunătățiți în următoarele 90 de zile; unde intră azi cererea și unde se blochează sau cere pe cineva să alerge după ea; cine e responsabil de pasul următor. Cu răspunsurile pregătesc harta și cele 3 soluții rapide. Apoi decidem împreună dacă are sens un Audit de Sisteme cu AI. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7681,7 +7681,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -7691,7 +7691,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. Companies in the US and China already run their operations on AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). I walked through the public journey of a {empresa} customer: {percurso}. Based only on what's public, I have a diagnostic hypothesis, not a conclusion: {pergunta} I've put it on a one-page mini-map and can implement 3 quick wins at no cost so we can test it. Who on the team would be the right person to validate it: operations, customer experience or digital transformation? A short exploratory call would be enough. I'll come prepared.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Empresas dos EUA e da China já conduzem as operações com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Percorri o percurso público de um cliente {empresa}: {percurso}. Com base no que é público, tenho uma hipótese de diagnóstico, não uma conclusão: {pergunta} Pus isto num mini-mapa de uma página e posso implementar sem custo 3 soluções rápidas para a testarmos. Quem na equipa seria a pessoa certa para o validar: operações, experiência do cliente ou transformação digital? Uma conversa exploratória curta chega. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -7713,7 +7713,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Following up on the mini-map of the {empresa} customer journey. I added one point: {valor} If you can point me to the right person, I'll send the map to them directly. I'll come prepared.</t>
+          <t>{saudacao} Volto ao mini-mapa sobre o percurso do cliente {empresa}. Acrescentei um único ponto: {valor} Se me puderem indicar a pessoa certa, envio-lhe o mapa diretamente. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7725,7 +7725,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -7735,19 +7735,19 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Thanks for getting back to me. To keep it short, three triage questions: which operational result do you want to improve in the next 90 days; where does a request come in today and where does it slow down or need someone chasing it; who owns the next step. With your answers I prepare the map and the 3 quick wins. Then we decide together whether an AI Systems Audit makes sense. I'll come prepared.</t>
+          <t>{saudacao} Obrigado pela resposta. Para não vos ocupar tempo, três perguntas curtas de triagem: que resultado operacional querem melhorar nos próximos 90 dias; onde entra hoje o pedido e onde abranda ou obriga alguém a correr atrás dele; quem é dono do próximo passo. Com as respostas preparo o mapa e as 3 soluções rápidas. Depois decidimos juntos se faz sentido uma Auditoria de Sistemas com IA. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -7757,19 +7757,19 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho}. Companii din SUA și China își conduc deja operațiunile cu sisteme AI cu reguli clare și cu un om la decizie; în România, doar 5% dintre firme folosesc AI (Eurostat, 2025). Voi aduceți cererea; noi lucrăm în stratul de după lead: cum ajunge cererea la echipă, ce context o însoțește, cine decide și cum se livrează. Nu înlocuim marketingul sau brandingul, protejăm rezultatul pe care îl generați deja. Am schițat o mini-hartă pentru un client tipic de-al vostru: {percurso}. Ca să vedeți cum lucrăm, implementăm fără cost 3 soluții rapide în propria voastră operațiune. Ați fi deschis la o întâlnire ca să vedem dacă are sens să lucrăm împreună? Voi fi pregătit.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. Companies in the US and China already run their operations on AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). I walked through the public journey of a {empresa} customer: {percurso}. Based only on what's public, I have a diagnostic hypothesis, not a conclusion: {pergunta} I've put it on a one-page mini-map and can implement 3 quick wins at no cost so we can test it. Who on the team would be the right person to validate it: operations, customer experience or digital transformation? A short exploratory call would be enough. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -7779,19 +7779,19 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu un exemplu concret de colaborare: {valor} Voi păstrați relația și serviciul, noi intrăm doar pe partea operațională. Voi fi pregătit.</t>
+          <t>{saudacao} Following up on the mini-map of the {empresa} customer journey. I added one point: {valor} If you can point me to the right person, I'll send the map to them directly. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -7801,7 +7801,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Mulțumesc pentru răspuns. Ca să nu vă ocup timpul, trei întrebări scurte de triaj: ce rezultat operațional vreți să îmbunătățiți în următoarele 90 de zile; unde intră azi cererea și unde se blochează sau cere pe cineva să alerge după ea; cine e responsabil de pasul următor. Cu răspunsurile pregătesc harta și cele 3 soluții rapide. Apoi decidem împreună dacă are sens un Audit de Sisteme cu AI. Voi fi pregătit.</t>
+          <t>{saudacao} Thanks for getting back to me. To keep it short, three triage questions: which operational result do you want to improve in the next 90 days; where does a request come in today and where does it slow down or need someone chasing it; who owns the next step. With your answers I prepare the map and the 3 quick wins. Then we decide together whether an AI Systems Audit makes sense. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -7813,7 +7813,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho}. Empresas dos EUA e da China já conduzem as operações com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Vocês trazem a procura; nós trabalhamos na camada depois do lead: como o pedido chega à equipa, que contexto leva, quem decide e como se entrega. Não substituímos o marketing nem a marca, protegemos o resultado que vocês já geram. Esbocei um mini-mapa para um cliente típico vosso: {percurso}. Para verem como trabalhamos, implementamos sem custo 3 soluções rápidas na vossa própria operação. Estariam abertos a uma reunião para ver se faz sentido trabalharmos juntos? Vou estar preparado.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho}. Companii din SUA și China își conduc deja operațiunile cu sisteme AI cu reguli clare și cu un om la decizie; în România, doar 5% dintre firme folosesc AI (Eurostat, 2025). Voi aduceți cererea; noi lucrăm în stratul de după lead: cum ajunge cererea la echipă, ce context o însoțește, cine decide și cum se livrează. Nu înlocuim marketingul sau brandingul, protejăm rezultatul pe care îl generați deja. Am schițat o mini-hartă pentru un client tipic de-al vostru: {percurso}. Ca să vedeți cum lucrăm, implementăm fără cost 3 soluții rapide în propria voastră operațiune. Ați fi deschis la o întâlnire ca să vedem dacă are sens să lucrăm împreună? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7835,7 +7835,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -7845,7 +7845,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto com um exemplo concreto de colaboração: {valor} Vocês mantêm a relação e o serviço, nós entramos só na parte operacional. Vou estar preparado.</t>
+          <t>{saudacao} Revin cu un exemplu concret de colaborare: {valor} Voi păstrați relația și serviciul, noi intrăm doar pe partea operațională. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -7867,7 +7867,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Obrigado pela resposta. Para não vos ocupar tempo, três perguntas curtas de triagem: que resultado operacional querem melhorar nos próximos 90 dias; onde entra hoje o pedido e onde abranda ou obriga alguém a correr atrás dele; quem é dono do próximo passo. Com as respostas preparo o mapa e as 3 soluções rápidas. Depois decidimos juntos se faz sentido uma Auditoria de Sistemas com IA. Vou estar preparado.</t>
+          <t>{saudacao} Mulțumesc pentru răspuns. Ca să nu vă ocup timpul, trei întrebări scurte de triaj: ce rezultat operațional vreți să îmbunătățiți în următoarele 90 de zile; unde intră azi cererea și unde se blochează sau cere pe cineva să alerge după ea; cine e responsabil de pasul următor. Cu răspunsurile pregătesc harta și cele 3 soluții rapide. Apoi decidem împreună dacă are sens un Audit de Sisteme cu AI. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7879,17 +7879,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho}. Companies in the US and China already run their operations on AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). You bring in the demand; we work on the layer after the lead: how the request reaches the team, what context travels with it, who decides and how it gets delivered. We don't replace marketing or branding, we protect the result you already generate. I sketched a mini-map for one of your typical clients: {percurso}. To show you how we work, we implement 3 quick wins in your own operation at no cost. Would you be open to a meeting to see whether it makes sense to work together? I'll come prepared.</t>
+          <t>{saudacao} Mă bucur că cele 3 soluții funcționează deja în echipa voastră. Vă propun un parteneriat simplu. Dacă vi se pare corect, menționați Pacheco Studios ca pe cei care v-au ajutat: o postare cu @pachecostudiospt și un rând pe site. Apoi, când un client de-al vostru se blochează după lead, ne faceți o introducere, cu acordul lui. Voi păstrați clientul și serviciul. Dacă ajungem să lucrăm cu acel client, primiți 10% din ce facturăm acolo, plătit la fiecare 3 luni, cât timp colaborarea continuă. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -7901,17 +7901,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Following up with one concrete collaboration example: {valor} You keep the relationship and the service; we only step into the operational side. I'll come prepared.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho}. Empresas dos EUA e da China já conduzem as operações com sistemas de IA com regras claras e uma pessoa na decisão; na Roménia, só 5% das empresas usam IA (Eurostat, 2025). Vocês trazem a procura; nós trabalhamos na camada depois do lead: como o pedido chega à equipa, que contexto leva, quem decide e como se entrega. Não substituímos o marketing nem a marca, protegemos o resultado que vocês já geram. Esbocei um mini-mapa para um cliente típico vosso: {percurso}. Para verem como trabalhamos, implementamos sem custo 3 soluções rápidas na vossa própria operação. Estariam abertos a uma reunião para ver se faz sentido trabalharmos juntos? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -7923,149 +7923,149 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Triagem (depois da resposta)</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Thanks for getting back to me. To keep it short, three triage questions: which operational result do you want to improve in the next 90 days; where does a request come in today and where does it slow down or need someone chasing it; who owns the next step. With your answers I prepare the map and the 3 quick wins. Then we decide together whether an AI Systems Audit makes sense. I'll come prepared.</t>
+          <t>{saudacao} Volto com um exemplo concreto de colaboração: {valor} Vocês mantêm a relação e o serviço, nós entramos só na parte operacional. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Punctul despre {tema} mi se pare esențial. În operațiunile pe care le analizez, întrebarea care schimbă cel mai mult este: {pergunta}</t>
+          <t>{saudacao} Obrigado pela resposta. Para não vos ocupar tempo, três perguntas curtas de triagem: que resultado operacional querem melhorar nos próximos 90 dias; onde entra hoje o pedido e onde abranda ou obriga alguém a correr atrás dele; quem é dono do próximo passo. Com as respostas preparo o mapa e as 3 soluções rápidas. Depois decidimos juntos se faz sentido uma Auditoria de Sistemas com IA. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Bună observație. Aș adăuga un detaliu din practică: {valor}</t>
+          <t>{saudacao} Fico contente por as 3 soluções já estarem a funcionar na vossa equipa. Proponho uma parceria simples. Se vos parecer justo, mencionem a Pacheco Studios como quem vos ajudou: um post com @pachecostudiospt e uma linha no site. Depois, quando um cliente vosso encravar depois do lead, apresentam-nos, com o acordo dele. Vocês mantêm o cliente e o serviço. Se chegarmos a trabalhar com esse cliente, recebem 10% do que faturamos lá, pago de 3 em 3 meses, enquanto a colaboração durar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>O întrebare sinceră pentru cei care au trecut prin asta: {pergunta}</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho}. Companies in the US and China already run their operations on AI systems with clear rules and a human at the decision point; in Romania, only 5% of companies use AI (Eurostat, 2025). You bring in the demand; we work on the layer after the lead: how the request reaches the team, what context travels with it, who decides and how it gets delivered. We don't replace marketing or branding, we protect the result you already generate. I sketched a mini-map for one of your typical clients: {percurso}. To show you how we work, we implement 3 quick wins in your own operation at no cost. Would you be open to a meeting to see whether it makes sense to work together? I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am comentat în ultimele săptămâni la postările voastre despre {tema}. Lucrez pe sisteme cu AI pentru operațiuni: unde stă contextul, cine răspunde de pasul următor și unde decide un om. Cred că publicul vostru ar găsi util un subiect ca acesta: {gancho}, ca articol, workshop scurt sau discuție la un eveniment. Ați fi deschis la o întâlnire scurtă? Voi fi pregătit.</t>
+          <t>{saudacao} Following up with one concrete collaboration example: {valor} You keep the relationship and the service; we only step into the operational side. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Triagem (depois da resposta)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu propunerea de subiect, acum mai concretă: {valor} Mă adaptez formatului care vă ajută cel mai mult. Voi fi pregătit.</t>
+          <t>{saudacao} Thanks for getting back to me. To keep it short, three triage questions: which operational result do you want to improve in the next 90 days; where does a request come in today and where does it slow down or need someone chasing it; who owns the next step. With your answers I prepare the map and the 3 quick wins. Then we decide together whether an AI Systems Audit makes sense. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>Parceria (depois dos 3 quick wins)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>O ponto sobre {tema} parece-me essencial. Nas operações que analiso, a pergunta que mais muda o resultado é: {pergunta}</t>
+          <t>{saudacao} Glad the 3 quick wins are already working for your team. I'd like to propose a simple partnership. If it feels fair, mention Pacheco Studios as the team that helped you: a post tagging @pachecostudiospt and a line on your site. Then, when one of your clients gets stuck after the lead, introduce us, with their consent. You keep the client and the service. If we end up working with that client, you get 10% of what we bill there, paid every 3 months for as long as the collaboration lasts. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -8077,17 +8077,17 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>Comentário: ponto</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Boa observação. Acrescentava um detalhe da prática: {valor}</t>
+          <t>Punctul despre {tema} mi se pare esențial. În operațiunile pe care le analizez, întrebarea care schimbă cel mai mult este: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -8099,17 +8099,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>Comentário: acréscimo</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Uma pergunta sincera para quem já passou por isto: {pergunta}</t>
+          <t>Bună observație. Aș adăuga un detaliu din practică: {valor}</t>
         </is>
       </c>
     </row>
@@ -8121,17 +8121,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Comentário: pergunta</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Tenho comentado nas vossas publicações sobre {tema}. Trabalho em sistemas com IA para operações: onde fica o contexto, quem é dono do próximo passo e onde decide uma pessoa. Acho que a vossa audiência ia achar útil um tema como este: {gancho}, em artigo, workshop curto ou conversa num evento. Estariam abertos a uma reunião curta? Vou estar preparado.</t>
+          <t>O întrebare sinceră pentru cei care au trecut prin asta: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -8143,17 +8143,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>DM 1</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto à proposta de tema, agora mais concreta: {valor} Adapto-me ao formato que mais vos ajudar. Vou estar preparado.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am comentat în ultimele săptămâni la postările voastre despre {tema}. Lucrez pe sisteme cu AI pentru operațiuni: unde stă contextul, cine răspunde de pasul următor și unde decide un om. Cred că publicul vostru ar găsi util un subiect ca acesta: {gancho}, ca articol, workshop scurt sau discuție la un eveniment. Ați fi deschis la o întâlnire scurtă? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -8165,17 +8165,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>The point about {tema} is key. In the operations I map, the question that changes the most is: {pergunta}</t>
+          <t>{saudacao} Revin cu propunerea de subiect, acum mai concretă: {valor} Mă adaptez formatului care vă ajută cel mai mult. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -8187,17 +8187,17 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>Comentário: ponto</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Good point. One detail from practice I'd add: {valor}</t>
+          <t>O ponto sobre {tema} parece-me essencial. Nas operações que analiso, a pergunta que mais muda o resultado é: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -8209,17 +8209,17 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>Comentário: acréscimo</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>An honest question for anyone who's been through this: {pergunta}</t>
+          <t>Boa observação. Acrescentava um detalhe da prática: {valor}</t>
         </is>
       </c>
     </row>
@@ -8231,17 +8231,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>DM 1</t>
+          <t>Comentário: pergunta</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I've been commenting on your posts about {tema}. I work on AI systems for operations: where context lives, who owns the next step and where a human decides. I think your audience would find a topic like this useful: {gancho}, as an article, a short workshop or a talk at an event. Would you be open to a short meeting? I'll come prepared.</t>
+          <t>Uma pergunta sincera para quem já passou por isto: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -8253,15 +8253,147 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>DM 1</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Tenho comentado nas vossas publicações sobre {tema}. Trabalho em sistemas com IA para operações: onde fica o contexto, quem é dono do próximo passo e onde decide uma pessoa. Acho que a vossa audiência ia achar útil um tema como este: {gancho}, em artigo, workshop curto ou conversa num evento. Estariam abertos a uma reunião curta? Vou estar preparado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>{saudacao} Volto à proposta de tema, agora mais concreta: {valor} Adapto-me ao formato que mais vos ajudar. Vou estar preparado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
           <t>en</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Comentário: ponto</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>The point about {tema} is key. In the operations I map, the question that changes the most is: {pergunta}</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Comentário: acréscimo</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Good point. One detail from practice I'd add: {valor}</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Comentário: pergunta</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>An honest question for anyone who's been through this: {pergunta}</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>DM 1</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I've been commenting on your posts about {tema}. I work on AI systems for operations: where context lives, who owns the next step and where a human decides. I think your audience would find a topic like this useful: {gancho}, as an article, a short workshop or a talk at an event. Would you be open to a short meeting? I'll come prepared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>{saudacao} Following up on the topic idea, now more concrete: {valor} Happy to fit whatever format helps you most. I'll come prepared.</t>
         </is>

</xml_diff>

<commit_message>
Instagram: contrapartida dos parceiros por ordem (testemunho logo nas quick wins) e mensagem «Testemunho»
- «Parceria» passa para antes de aplicar os 3 quick wins: incentivo primeiro (15 % + 5 % trimestral), depois proposta assinada
- Contrapartida por ordem (decisão do Tomás, 14h44): testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês
- Mensagem «Testemunho» nova (RO, PT, EN; influenciador e PME)
- Aviso no gerador: «Parceria» e «Testemunho» só com @ e texto confirmados pelo Tomás

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bCka4TNe6PKPBEx4M62DX
</commit_message>
<xml_diff>
--- a/research/instagram/prospecao-instagram.xlsx
+++ b/research/instagram/prospecao-instagram.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; indicações consentidas depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% de 3 em 3 meses; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; indicações consentidas depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% de 3 em 3 meses; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
         </is>
       </c>
       <c r="O3" s="2" t="n">
@@ -974,7 +974,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; indicações consentidas depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% de 3 em 3 meses; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
         </is>
       </c>
       <c r="O4" s="2" t="n">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; indicações consentidas depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% de 3 em 3 meses; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
         </is>
       </c>
       <c r="O5" s="2" t="n">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O7" s="2" t="n">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O8" s="2" t="n">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O9" s="2" t="n">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O10" s="2" t="n">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O11" s="2" t="n">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O12" s="2" t="n">
@@ -9593,7 +9593,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; indicações consentidas depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% de 3 em 3 meses; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -9667,7 +9667,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; indicações e co-entrega depois: 15% da implementação + 5% de 3 em 3 meses enquanto trabalharmos com o indicado.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -9724,7 +9724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9878,12 +9878,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>Parceria (antes de aplicar os 3 quick wins: incentivo primeiro)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Mă bucur că cele 3 soluții merg deja la tine. Am o propunere simplă de parteneriat, și încep cu partea care contează pentru tine: când întâlnești o afacere care se blochează în același loc, ne faci o introducere, cu acordul ei. Dacă ajungem să lucrăm cu acea afacere, primești 15% din valoarea implementării și apoi 5% la fiecare 3 luni, cât timp lucrăm cu ea. Valoarea depinde de afacere: la o firmă mai mare, implementarea e mai mare, și la fel partea ta. Dacă ți se pare corect, îți trimit propunerea scrisă, cu regulile simple: un testimonial de la tine și o postare pe lună despre noi, cu @pachecostudiospt. Voi fi pregătit.</t>
+          <t>{saudacao} Înainte să aplicăm cele 3 soluții, vreau să-ți arăt ce poți câștiga dacă lucrăm și mai departe împreună. Când ne prezinți o afacere care se blochează în același loc, cu acordul ei, și ajungem să lucrăm cu ea, primești 15% din valoarea implementării și apoi 5% la fiecare 3 luni, cât timp lucrăm cu ea. Valoarea depinde de afacere: cu cât firma e mai mare, cu atât implementarea e mai mare, și la fel partea ta. În schimb îți cerem trei lucruri, în ordinea asta: în ziua în care cele 3 soluții funcționează, un prim testimonial online și o recomandare, ca mulțumire; apoi recomandări din gură în gură; apoi o mențiune pe lună în conținutul tău. Dacă ți se pare corect, îți trimit propunerea scrisă, de semnat. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -9895,17 +9895,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>Testemunho (no dia em que os 3 quick wins ficam a funcionar)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho} e olhei para o percurso público: {percurso}. Não tenho acesso ao interior, por isso não presumo nenhum problema. A pergunta que validaria: {pergunta} {isca} As empresas dos EUA e da China já trabalham assim; na Roménia, 5% das empresas (Eurostat, 2025). Se não, faz uma triagem connosco: preparei uma página (Micro System Print) com o que validaria e uma solução rápida que podes aplicar já, e validamo-la juntos. Vou estar preparado.</t>
+          <t>{saudacao} Cele 3 soluții funcționează de azi. Mulțumesc pentru încredere. Cum am vorbit, dacă ești mulțumit, un prim testimonial online ar însemna mult pentru noi: o postare sau un story cu @pachecostudiospt, în cuvintele tale, despre ce s-a schimbat, și o recomandare. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -9922,12 +9922,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>D4: observação nova</t>
+          <t>D0: DM 1</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto com uma única observação, não com uma oferta: {valor} A pergunta que validaria contigo: o que acontece a um pedido depois de entrar? A página está pronta; se quiseres, faz uma triagem connosco. Vou estar preparado.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho} e olhei para o percurso público: {percurso}. Não tenho acesso ao interior, por isso não presumo nenhum problema. A pergunta que validaria: {pergunta} {isca} As empresas dos EUA e da China já trabalham assim; na Roménia, 5% das empresas (Eurostat, 2025). Se não, faz uma triagem connosco: preparei uma página (Micro System Print) com o que validaria e uma solução rápida que podes aplicar já, e validamo-la juntos. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -9944,12 +9944,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>D7: pergunta sim ou não</t>
+          <t>D4: observação nova</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Uma pergunta simples, para não te ocupar: este passo já está resolvido de ponta a ponta aí, ou vale a pena validarmos o mapa juntos? Um sim ou um não chega. Vou estar preparado.</t>
+          <t>{saudacao} Volto com uma única observação, não com uma oferta: {valor} A pergunta que validaria contigo: o que acontece a um pedido depois de entrar? A página está pronta; se quiseres, faz uma triagem connosco. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -9966,12 +9966,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>D12: fecho limpo</t>
+          <t>D7: pergunta sim ou não</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Fecho o assunto por agora. Deixo-te o Micro System Print; se este ponto se tornar prioridade, validamos o mapa quando quiseres. Vou estar preparado.</t>
+          <t>{saudacao} Uma pergunta simples, para não te ocupar: este passo já está resolvido de ponta a ponta aí, ou vale a pena validarmos o mapa juntos? Um sim ou um não chega. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -9988,12 +9988,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Triagem (quando respondem, com o Micro System Print)</t>
+          <t>D12: fecho limpo</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Obrigado pela resposta. Envio-te o Micro System Print de uma página: o percurso público que vi, o passo marcado «a validar» e o fluxo que proporia, com dono, regra e passagem a uma pessoa. Não afirmo que tens um problema: é a primeira coisa que validaria. Fazemos a triagem juntos, numa conversa curta em que eu conduzo as perguntas, sem formulários. Se o mapa se confirmar, implementamos 3 soluções rápidas, sem custo, para veres como trabalhamos; o passo seguinte é a Auditoria de Sistemas com IA, creditada na implementação. Se não se confirmar, a página fica contigo como referência. Quando te dá jeito? Vou estar preparado.</t>
+          <t>{saudacao} Fecho o assunto por agora. Deixo-te o Micro System Print; se este ponto se tornar prioridade, validamos o mapa quando quiseres. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10010,12 +10010,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>Triagem (quando respondem, com o Micro System Print)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Fico contente por as 3 soluções já estarem a funcionar contigo. Tenho uma proposta simples de parceria, e começo pela parte que te interessa: quando conheceres um negócio que encrava no mesmo sítio, apresentas-nos, com o acordo dele. Se chegarmos a trabalhar com esse negócio, recebes 15% do valor da implementação e depois 5% de 3 em 3 meses, enquanto trabalharmos com ele. O valor depende do negócio: numa empresa maior, a implementação é maior, e a tua parte também. Se te parecer justo, envio-te a proposta escrita, com as regras simples: um testemunho teu e um post por mês sobre nós, com @pachecostudiospt. Vou estar preparado.</t>
+          <t>{saudacao} Obrigado pela resposta. Envio-te o Micro System Print de uma página: o percurso público que vi, o passo marcado «a validar» e o fluxo que proporia, com dono, regra e passagem a uma pessoa. Não afirmo que tens um problema: é a primeira coisa que validaria. Fazemos a triagem juntos, numa conversa curta em que eu conduzo as perguntas, sem formulários. Se o mapa se confirmar, implementamos 3 soluções rápidas, sem custo, para veres como trabalhamos; o passo seguinte é a Auditoria de Sistemas com IA, creditada na implementação. Se não se confirmar, a página fica contigo como referência. Quando te dá jeito? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10027,17 +10027,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>Parceria (antes de aplicar os 3 quick wins: incentivo primeiro)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho} and looked at the public journey: {percurso}. I can't see the inside, so I'm not assuming a problem. The question I'd validate: {pergunta} {isca} Companies in the US and China already work this way; in Romania, 5% of companies do (Eurostat, 2025). If not, run a triage with us: I've prepared a page (Micro System Print) with what I'd validate and a quick win you can apply right away, and we validate it together. I'll come prepared.</t>
+          <t>{saudacao} Antes de aplicarmos as 3 soluções, quero mostrar-te o que podes ganhar se continuarmos a trabalhar juntos. Quando nos apresentares um negócio que encrava no mesmo sítio, com o acordo dele, e chegarmos a trabalhar com ele, recebes 15% do valor da implementação e depois 5% de 3 em 3 meses, enquanto trabalharmos com ele. O valor depende do negócio: quanto maior a empresa, maior a implementação, e maior a tua parte. Em troca pedimos três coisas, por esta ordem: no dia em que as 3 soluções ficam a funcionar, um primeiro testemunho online e uma recomendação, como agradecimento; depois, recomendações boca a boca; depois, uma menção por mês nos teus conteúdos. Se te parecer justo, envio a proposta escrita para assinar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10049,17 +10049,17 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>D4: observação nova</t>
+          <t>Testemunho (no dia em que os 3 quick wins ficam a funcionar)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Back with a single observation, not an offer: {valor} The question I'd validate with you: what happens to a request after it comes in? The page is ready; if you want, run a triage with us. I'll come prepared.</t>
+          <t>{saudacao} As 3 soluções estão a funcionar desde hoje. Obrigado pela confiança. Como combinámos, se estiveres satisfeito, um primeiro testemunho online significava muito para nós: um post ou story com @pachecostudiospt, nas tuas palavras, sobre o que mudou, e uma recomendação. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10076,12 +10076,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>D7: pergunta sim ou não</t>
+          <t>D0: DM 1</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} One simple question, so I don't take your time: is this step already solved end to end on your side, or is it worth validating the map together? A yes or a no is enough. I'll come prepared.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho} and looked at the public journey: {percurso}. I can't see the inside, so I'm not assuming a problem. The question I'd validate: {pergunta} {isca} Companies in the US and China already work this way; in Romania, 5% of companies do (Eurostat, 2025). If not, run a triage with us: I've prepared a page (Micro System Print) with what I'd validate and a quick win you can apply right away, and we validate it together. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -10098,12 +10098,12 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>D12: fecho limpo</t>
+          <t>D4: observação nova</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Closing this for now. I'll leave the Micro System Print with you; if this point becomes a priority, we validate the map whenever suits you. I'll come prepared.</t>
+          <t>{saudacao} Back with a single observation, not an offer: {valor} The question I'd validate with you: what happens to a request after it comes in? The page is ready; if you want, run a triage with us. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -10120,12 +10120,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Triagem (quando respondem, com o Micro System Print)</t>
+          <t>D7: pergunta sim ou não</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Thanks for getting back to me. I'm sending you the one-page Micro System Print: the public journey I saw, the step marked "to validate" and the flow I'd propose, with an owner, a rule and a human handoff. I'm not claiming you have a problem: it's the first thing I would validate. We run the triage together, in a short call where I lead the questions, no forms. If the map holds, we implement 3 quick wins at no cost so you see how we work; the next step is the AI Systems Audit, credited against implementation. If it doesn't hold, the page stays with you as a reference. When suits you? I'll come prepared.</t>
+          <t>{saudacao} One simple question, so I don't take your time: is this step already solved end to end on your side, or is it worth validating the map together? A yes or a no is enough. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -10142,78 +10142,78 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>D12: fecho limpo</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Glad the 3 quick wins are already working for you. I have a simple partnership proposal, starting with the part that matters to you: when you meet a business stuck in the same place, introduce us, with their consent. If we end up working with that business, you get 15% of the implementation value and then 5% every 3 months for as long as we work with them. The value depends on the business: a bigger company means a bigger implementation, and a bigger share for you. If that feels fair, I'll send you the written proposal with the simple rules: a testimonial from you and one post a month about us, tagging @pachecostudiospt. I'll come prepared.</t>
+          <t>{saudacao} Closing this for now. I'll leave the Micro System Print with you; if this point becomes a priority, we validate the map whenever suits you. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Grande negócio</t>
+          <t>Influenciador / operador</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>Triagem (quando respondem, com o Micro System Print)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am parcurs traseul public al unui client {empresa}: {percurso}. Nu am acces la operațiunea internă, deci nu presupun nicio problemă. Întrebarea pe care aș valida-o: {pergunta} {isca} Companiile din SUA și China lucrează deja așa; în România, 5% dintre firme (Eurostat, 2025). Am pregătit o pagină (Micro System Print) cu ce aș valida. Dacă nu e rezolvat cap-coadă, faceți un triaj cu noi: cine ar fi persoana potrivită, din operațiuni, experiența clienților sau transformare digitală? Voi fi pregătit.</t>
+          <t>{saudacao} Thanks for getting back to me. I'm sending you the one-page Micro System Print: the public journey I saw, the step marked "to validate" and the flow I'd propose, with an owner, a rule and a human handoff. I'm not claiming you have a problem: it's the first thing I would validate. We run the triage together, in a short call where I lead the questions, no forms. If the map holds, we implement 3 quick wins at no cost so you see how we work; the next step is the AI Systems Audit, credited against implementation. If it doesn't hold, the page stays with you as a reference. When suits you? I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Grande negócio</t>
+          <t>Influenciador / operador</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>D4: observação nova</t>
+          <t>Parceria (antes de aplicar os 3 quick wins: incentivo primeiro)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu o singură observație despre traseul clientului {empresa}, nu cu o ofertă: {valor} Întrebarea pe care aș valida-o: după ce o cerere intră, cine rămâne responsabil până la confirmare? Dacă îmi puteți indica persoana potrivită, îi trimit direct pagina. Voi fi pregătit.</t>
+          <t>{saudacao} Before we apply the 3 quick wins, I want to show you what you can earn if we keep working together. When you introduce us to a business stuck in the same place, with their consent, and we end up working with them, you get 15% of the implementation value and then 5% every 3 months for as long as we work with them. The value depends on the business: the bigger the company, the bigger the implementation, and the bigger your share. In return we ask for three things, in this order: on the day the 3 quick wins go live, a first online testimonial and a recommendation, as a thank-you; then word-of-mouth recommendations; then one mention a month in your content. If that feels fair, I'll send the written proposal to sign. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Grande negócio</t>
+          <t>Influenciador / operador</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>D7: pergunta sim ou não</t>
+          <t>Testemunho (no dia em que os 3 quick wins ficam a funcionar)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} O întrebare simplă, ca să nu vă ocup timpul: pasul acesta e deja rezolvat cap-coadă la {empresa}, sau merită o validare scurtă cu persoana responsabilă? Un da sau un nu e suficient. Voi fi pregătit.</t>
+          <t>{saudacao} The 3 quick wins are live as of today. Thank you for the trust. As agreed, if you're happy, a first online testimonial would mean a lot to us: a post or story tagging @pachecostudiospt, in your own words, about what changed, plus a recommendation. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -10230,12 +10230,12 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>D12: fecho limpo</t>
+          <t>D0: DM 1</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Închid subiectul pentru acum. Vă las Micro System Print-ul despre traseul clientului {empresa}; dacă punctul acesta devine prioritate, validăm harta cu persoana potrivită. Voi fi pregătit.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am parcurs traseul public al unui client {empresa}: {percurso}. Nu am acces la operațiunea internă, deci nu presupun nicio problemă. Întrebarea pe care aș valida-o: {pergunta} {isca} Companiile din SUA și China lucrează deja așa; în România, 5% dintre firme (Eurostat, 2025). Am pregătit o pagină (Micro System Print) cu ce aș valida. Dacă nu e rezolvat cap-coadă, faceți un triaj cu noi: cine ar fi persoana potrivită, din operațiuni, experiența clienților sau transformare digitală? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10252,12 +10252,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Triagem (quando respondem, com o Micro System Print)</t>
+          <t>D4: observação nova</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Mulțumesc pentru răspuns. Vă trimit Micro System Print-ul de o pagină: traseul public al unui client {empresa}, pasul marcat „de validat” și fluxul pe care l-aș propune, cu responsabil, regulă și predare la om. Nu afirm că există o problemă: e primul lucru pe care l-aș valida. Propun un triaj condus de noi, într-o întâlnire scurtă cu persoana care cunoaște traseul, fără formulare. Dacă harta se confirmă, alegem împreună 3 soluții rapide, fără cost, ca să o testăm; pasul următor e Auditul de Sisteme cu AI, creditat în implementare. Dacă nu, pagina rămâne ca referință. Cui i-ar fi cel mai util să ajungă? Voi fi pregătit.</t>
+          <t>{saudacao} Revin cu o singură observație despre traseul clientului {empresa}, nu cu o ofertă: {valor} Întrebarea pe care aș valida-o: după ce o cerere intră, cine rămâne responsabil până la confirmare? Dacă îmi puteți indica persoana potrivită, îi trimit direct pagina. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10269,17 +10269,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>D7: pergunta sim ou não</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Percorri o percurso público de um cliente {empresa}: {percurso}. Não tenho acesso à operação interna, por isso não presumo nenhum problema. A pergunta que validaria: {pergunta} {isca} As empresas dos EUA e da China já trabalham assim; na Roménia, 5% das empresas (Eurostat, 2025). Preparei uma página (Micro System Print) com o que validaria. Se não estiver resolvido de ponta a ponta, façam uma triagem connosco: quem seria a pessoa certa, em operações, experiência do cliente ou transformação digital? Vou estar preparado.</t>
+          <t>{saudacao} O întrebare simplă, ca să nu vă ocup timpul: pasul acesta e deja rezolvat cap-coadă la {empresa}, sau merită o validare scurtă cu persoana responsabilă? Un da sau un nu e suficient. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10291,17 +10291,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>D4: observação nova</t>
+          <t>D12: fecho limpo</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto com uma única observação sobre o percurso do cliente {empresa}, não com uma oferta: {valor} A pergunta que validaria: depois de um pedido entrar, quem fica dono dele até à confirmação? Se me indicarem a pessoa certa, envio-lhe a página diretamente. Vou estar preparado.</t>
+          <t>{saudacao} Închid subiectul pentru acum. Vă las Micro System Print-ul despre traseul clientului {empresa}; dacă punctul acesta devine prioritate, validăm harta cu persoana potrivită. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10313,17 +10313,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>D7: pergunta sim ou não</t>
+          <t>Triagem (quando respondem, com o Micro System Print)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Uma pergunta simples, para não vos ocupar: este passo já está resolvido de ponta a ponta na {empresa}, ou vale uma validação curta com a pessoa responsável? Um sim ou um não chega. Vou estar preparado.</t>
+          <t>{saudacao} Mulțumesc pentru răspuns. Vă trimit Micro System Print-ul de o pagină: traseul public al unui client {empresa}, pasul marcat „de validat” și fluxul pe care l-aș propune, cu responsabil, regulă și predare la om. Nu afirm că există o problemă: e primul lucru pe care l-aș valida. Propun un triaj condus de noi, într-o întâlnire scurtă cu persoana care cunoaște traseul, fără formulare. Dacă harta se confirmă, alegem împreună 3 soluții rapide, fără cost, ca să o testăm; pasul următor e Auditul de Sisteme cu AI, creditat în implementare. Dacă nu, pagina rămâne ca referință. Cui i-ar fi cel mai util să ajungă? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10340,12 +10340,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>D12: fecho limpo</t>
+          <t>D0: DM 1</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Fecho o assunto por agora. Deixo-vos o Micro System Print sobre o percurso do cliente {empresa}; se este ponto se tornar prioridade, validamos o mapa com a pessoa certa. Vou estar preparado.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Percorri o percurso público de um cliente {empresa}: {percurso}. Não tenho acesso à operação interna, por isso não presumo nenhum problema. A pergunta que validaria: {pergunta} {isca} As empresas dos EUA e da China já trabalham assim; na Roménia, 5% das empresas (Eurostat, 2025). Preparei uma página (Micro System Print) com o que validaria. Se não estiver resolvido de ponta a ponta, façam uma triagem connosco: quem seria a pessoa certa, em operações, experiência do cliente ou transformação digital? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10362,12 +10362,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Triagem (quando respondem, com o Micro System Print)</t>
+          <t>D4: observação nova</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Obrigado pela resposta. Envio o Micro System Print de uma página: o percurso público de um cliente {empresa}, o passo marcado «a validar» e o fluxo que proporia, com dono, regra e passagem a uma pessoa. Não afirmo que existe um problema: é a primeira coisa que validaria. Proponho uma triagem conduzida por nós, numa conversa curta com quem conhece o percurso, sem formulários. Se o mapa se confirmar, escolhemos juntos 3 soluções rápidas, sem custo, para o testar; o passo seguinte é a Auditoria de Sistemas com IA, creditada na implementação. Se não, a página fica como referência. A quem seria mais útil chegar? Vou estar preparado.</t>
+          <t>{saudacao} Volto com uma única observação sobre o percurso do cliente {empresa}, não com uma oferta: {valor} A pergunta que validaria: depois de um pedido entrar, quem fica dono dele até à confirmação? Se me indicarem a pessoa certa, envio-lhe a página diretamente. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10379,17 +10379,17 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>D7: pergunta sim ou não</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I walked through the public journey of a {empresa} customer: {percurso}. I can't see the internal operation, so I'm not assuming a problem. The question I'd validate: {pergunta} {isca} Companies in the US and China already work this way; in Romania, 5% of companies do (Eurostat, 2025). I've prepared a page (Micro System Print) with what I'd validate. If it isn't solved end to end, run a triage with us: who would be the right person, in operations, customer experience or digital transformation? I'll come prepared.</t>
+          <t>{saudacao} Uma pergunta simples, para não vos ocupar: este passo já está resolvido de ponta a ponta na {empresa}, ou vale uma validação curta com a pessoa responsável? Um sim ou um não chega. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10401,17 +10401,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>D4: observação nova</t>
+          <t>D12: fecho limpo</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Back with a single observation about the {empresa} customer journey, not an offer: {valor} The question I'd validate: after a request comes in, who owns it until it's confirmed? If you can point me to the right person, I'll send them the page directly. I'll come prepared.</t>
+          <t>{saudacao} Fecho o assunto por agora. Deixo-vos o Micro System Print sobre o percurso do cliente {empresa}; se este ponto se tornar prioridade, validamos o mapa com a pessoa certa. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10423,17 +10423,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>D7: pergunta sim ou não</t>
+          <t>Triagem (quando respondem, com o Micro System Print)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} One simple question, so I don't take your time: is this step already solved end to end at {empresa}, or is it worth a short validation with the person in charge? A yes or a no is enough. I'll come prepared.</t>
+          <t>{saudacao} Obrigado pela resposta. Envio o Micro System Print de uma página: o percurso público de um cliente {empresa}, o passo marcado «a validar» e o fluxo que proporia, com dono, regra e passagem a uma pessoa. Não afirmo que existe um problema: é a primeira coisa que validaria. Proponho uma triagem conduzida por nós, numa conversa curta com quem conhece o percurso, sem formulários. Se o mapa se confirmar, escolhemos juntos 3 soluções rápidas, sem custo, para o testar; o passo seguinte é a Auditoria de Sistemas com IA, creditada na implementação. Se não, a página fica como referência. A quem seria mais útil chegar? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10450,12 +10450,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>D12: fecho limpo</t>
+          <t>D0: DM 1</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Closing this for now. I'll leave the Micro System Print on the {empresa} customer journey with you; if this point becomes a priority, we validate the map with the right person. I'll come prepared.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I walked through the public journey of a {empresa} customer: {percurso}. I can't see the internal operation, so I'm not assuming a problem. The question I'd validate: {pergunta} {isca} Companies in the US and China already work this way; in Romania, 5% of companies do (Eurostat, 2025). I've prepared a page (Micro System Print) with what I'd validate. If it isn't solved end to end, run a triage with us: who would be the right person, in operations, customer experience or digital transformation? I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -10472,78 +10472,78 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Triagem (quando respondem, com o Micro System Print)</t>
+          <t>D4: observação nova</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Thanks for getting back to me. I'm sending the one-page Micro System Print: the public journey of a {empresa} customer, the step marked "to validate" and the flow I'd propose, with an owner, a rule and a human handoff. I'm not claiming there is a problem: it's the first thing I would validate. I propose a triage led by us, in a short call with the person who knows the journey, no forms. If the map holds, we pick 3 quick wins together, at no cost, to test it; the next step is the AI Systems Audit, credited against implementation. If not, the page stays as a reference. Who would it be most useful to reach? I'll come prepared.</t>
+          <t>{saudacao} Back with a single observation about the {empresa} customer journey, not an offer: {valor} The question I'd validate: after a request comes in, who owns it until it's confirmed? If you can point me to the right person, I'll send them the page directly. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>D7: pergunta sim ou não</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho}. Voi aduceți cererea; noi lucrăm în stratul de după lead. Traseul unui client tipic de-al vostru: {percurso}. Nu presupun nicio problemă; întrebarea pe care aș valida-o: {pergunta} {isca} Companiile din SUA și China lucrează deja așa; în România, 5% dintre firme (Eurostat, 2025). Dacă nu, faceți un triaj cu noi: am pregătit o pagină (Micro System Print) cu ce aș valida și o soluție rapidă aplicabilă imediat, și o validăm împreună. Voi fi pregătit.</t>
+          <t>{saudacao} One simple question, so I don't take your time: is this step already solved end to end at {empresa}, or is it worth a short validation with the person in charge? A yes or a no is enough. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>D4: observação nova</t>
+          <t>D12: fecho limpo</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu o singură observație, nu cu o ofertă: {valor} Voi păstrați relația și serviciul; noi intrăm doar pe partea operațională. Dacă are sens, faceți un triaj cu noi: pagina e gata. Voi fi pregătit.</t>
+          <t>{saudacao} Closing this for now. I'll leave the Micro System Print on the {empresa} customer journey with you; if this point becomes a priority, we validate the map with the right person. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>PME / parceiro de indicação</t>
+          <t>Grande negócio</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>D7: pergunta sim ou não</t>
+          <t>Triagem (quando respondem, com o Micro System Print)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} O întrebare simplă, ca să nu vă ocup timpul: pasul de după lead e deja rezolvat cap-coadă la clienții voștri, sau merită să validăm harta împreună? Un da sau un nu e suficient. Voi fi pregătit.</t>
+          <t>{saudacao} Thanks for getting back to me. I'm sending the one-page Micro System Print: the public journey of a {empresa} customer, the step marked "to validate" and the flow I'd propose, with an owner, a rule and a human handoff. I'm not claiming there is a problem: it's the first thing I would validate. I propose a triage led by us, in a short call with the person who knows the journey, no forms. If the map holds, we pick 3 quick wins together, at no cost, to test it; the next step is the AI Systems Audit, credited against implementation. If not, the page stays as a reference. Who would it be most useful to reach? I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -10560,12 +10560,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>D12: fecho limpo</t>
+          <t>D0: DM 1</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Închid subiectul pentru acum. Vă las Micro System Print-ul; dacă punctul acesta devine prioritate pentru voi sau pentru un client, validăm harta împreună. Voi fi pregătit.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am văzut {gancho}. Voi aduceți cererea; noi lucrăm în stratul de după lead. Traseul unui client tipic de-al vostru: {percurso}. Nu presupun nicio problemă; întrebarea pe care aș valida-o: {pergunta} {isca} Companiile din SUA și China lucrează deja așa; în România, 5% dintre firme (Eurostat, 2025). Dacă nu, faceți un triaj cu noi: am pregătit o pagină (Micro System Print) cu ce aș valida și o soluție rapidă aplicabilă imediat, și o validăm împreună. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10582,12 +10582,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Triagem (quando respondem, com o Micro System Print)</t>
+          <t>D4: observação nova</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Mulțumesc pentru răspuns. Vă trimit Micro System Print-ul de o pagină: traseul unui client tipic de-al vostru, pasul marcat „de validat” și fluxul pe care l-aș propune, cu responsabil, regulă și predare la om. Nu afirm că există o problemă: e primul lucru pe care l-aș valida. Facem triajul împreună, într-o întâlnire scurtă în care conduc eu întrebările, fără formulare. Dacă harta se confirmă, implementăm 3 soluții rapide, fără cost, în operațiunea voastră, ca să vedeți cum lucrăm; pasul următor e Auditul de Sisteme cu AI, creditat în implementare, la voi sau la un client. Dacă nu se confirmă, pagina rămâne ca referință. Când v-ar conveni? Voi fi pregătit.</t>
+          <t>{saudacao} Revin cu o singură observație, nu cu o ofertă: {valor} Voi păstrați relația și serviciul; noi intrăm doar pe partea operațională. Dacă are sens, faceți un triaj cu noi: pagina e gata. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10604,12 +10604,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>D7: pergunta sim ou não</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Mă bucur că cele 3 soluții funcționează deja în echipa voastră. Vă propun un parteneriat simplu și încep cu partea care contează pentru voi: când un client de-al vostru se blochează după lead, ne faceți o introducere, cu acordul lui. Voi păstrați clientul și serviciul. Dacă ajungem să lucrăm cu acel client, primiți 15% din valoarea implementării și apoi 5% la fiecare 3 luni, cât timp lucrăm cu el. Valoarea depinde de client: la o firmă mai mare, implementarea e mai mare, și la fel partea voastră. Dacă vi se pare corect, vă trimit propunerea scrisă, cu regulile simple: un testimonial din partea voastră și o postare pe lună despre noi, cu @pachecostudiospt. Voi fi pregătit.</t>
+          <t>{saudacao} O întrebare simplă, ca să nu vă ocup timpul: pasul de după lead e deja rezolvat cap-coadă la clienții voștri, sau merită să validăm harta împreună? Un da sau un nu e suficient. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10621,17 +10621,17 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>D12: fecho limpo</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho}. Vocês trazem a procura; nós trabalhamos na camada depois do lead. O percurso de um cliente típico vosso: {percurso}. Não presumo nenhum problema; a pergunta que validaria: {pergunta} {isca} As empresas dos EUA e da China já trabalham assim; na Roménia, 5% das empresas (Eurostat, 2025). Se não, façam uma triagem connosco: preparei uma página (Micro System Print) com o que validaria e uma solução rápida aplicável já, e validamo-la juntos. Vou estar preparado.</t>
+          <t>{saudacao} Închid subiectul pentru acum. Vă las Micro System Print-ul; dacă punctul acesta devine prioritate pentru voi sau pentru un client, validăm harta împreună. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10643,17 +10643,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>D4: observação nova</t>
+          <t>Triagem (quando respondem, com o Micro System Print)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto com uma única observação, não com uma oferta: {valor} Vocês mantêm a relação e o serviço; nós entramos só na parte operacional. Se fizer sentido, façam uma triagem connosco: a página está pronta. Vou estar preparado.</t>
+          <t>{saudacao} Mulțumesc pentru răspuns. Vă trimit Micro System Print-ul de o pagină: traseul unui client tipic de-al vostru, pasul marcat „de validat” și fluxul pe care l-aș propune, cu responsabil, regulă și predare la om. Nu afirm că există o problemă: e primul lucru pe care l-aș valida. Facem triajul împreună, într-o întâlnire scurtă în care conduc eu întrebările, fără formulare. Dacă harta se confirmă, implementăm 3 soluții rapide, fără cost, în operațiunea voastră, ca să vedeți cum lucrăm; pasul următor e Auditul de Sisteme cu AI, creditat în implementare, la voi sau la un client. Dacă nu se confirmă, pagina rămâne ca referință. Când v-ar conveni? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10665,17 +10665,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>D7: pergunta sim ou não</t>
+          <t>Parceria (antes de aplicar os 3 quick wins: incentivo primeiro)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Uma pergunta simples, para não vos ocupar: o passo depois do lead já está resolvido de ponta a ponta nos vossos clientes, ou vale a pena validarmos o mapa juntos? Um sim ou um não chega. Vou estar preparado.</t>
+          <t>{saudacao} Înainte să aplicăm cele 3 soluții, vreau să vă arăt ce puteți câștiga dacă lucrăm și mai departe împreună. Când un client de-al vostru se blochează după lead și ne faceți o introducere, cu acordul lui, voi păstrați clientul și serviciul. Dacă ajungem să lucrăm cu el, primiți 15% din valoarea implementării și apoi 5% la fiecare 3 luni, cât timp lucrăm cu el. Valoarea depinde de client: cu cât firma e mai mare, cu atât implementarea e mai mare, și la fel partea voastră. În schimb vă cerem trei lucruri, în ordinea asta: în ziua în care cele 3 soluții funcționează, un prim testimonial online și o recomandare, ca mulțumire; apoi recomandări din gură în gură; apoi o mențiune pe lună în conținutul vostru. Dacă vi se pare corect, vă trimit propunerea scrisă, de semnat. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10687,17 +10687,17 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>D12: fecho limpo</t>
+          <t>Testemunho (no dia em que os 3 quick wins ficam a funcionar)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Fecho o assunto por agora. Deixo-vos o Micro System Print; se este ponto se tornar prioridade para vocês ou para um cliente, validamos o mapa juntos. Vou estar preparado.</t>
+          <t>{saudacao} Cele 3 soluții funcționează de azi în echipa voastră. Mulțumesc pentru încredere. Cum am vorbit, dacă sunteți mulțumiți, un prim testimonial online ar însemna mult pentru noi: o postare cu @pachecostudiospt, în cuvintele voastre, despre ce s-a schimbat, și o recomandare. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10714,12 +10714,12 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Triagem (quando respondem, com o Micro System Print)</t>
+          <t>D0: DM 1</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Obrigado pela resposta. Envio o Micro System Print de uma página: o percurso de um cliente típico vosso, o passo marcado «a validar» e o fluxo que proporia, com dono, regra e passagem a uma pessoa. Não afirmo que existe um problema: é a primeira coisa que validaria. Fazemos a triagem juntos, numa conversa curta em que eu conduzo as perguntas, sem formulários. Se o mapa se confirmar, implementamos 3 soluções rápidas, sem custo, na vossa operação, para verem como trabalhamos; o passo seguinte é a Auditoria de Sistemas com IA, creditada na implementação, em vocês ou num cliente. Se não se confirmar, a página fica como referência. Quando vos dá jeito? Vou estar preparado.</t>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Vi {gancho}. Vocês trazem a procura; nós trabalhamos na camada depois do lead. O percurso de um cliente típico vosso: {percurso}. Não presumo nenhum problema; a pergunta que validaria: {pergunta} {isca} As empresas dos EUA e da China já trabalham assim; na Roménia, 5% das empresas (Eurostat, 2025). Se não, façam uma triagem connosco: preparei uma página (Micro System Print) com o que validaria e uma solução rápida aplicável já, e validamo-la juntos. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10736,12 +10736,12 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>D4: observação nova</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Fico contente por as 3 soluções já estarem a funcionar na vossa equipa. Proponho uma parceria simples e começo pela parte que vos interessa: quando um cliente vosso encravar depois do lead, apresentam-nos, com o acordo dele. Vocês mantêm o cliente e o serviço. Se chegarmos a trabalhar com esse cliente, recebem 15% do valor da implementação e depois 5% de 3 em 3 meses, enquanto trabalharmos com ele. O valor depende do cliente: numa empresa maior, a implementação é maior, e a vossa parte também. Se vos parecer justo, envio a proposta escrita, com as regras simples: um testemunho vosso e um post por mês sobre nós, com @pachecostudiospt. Vou estar preparado.</t>
+          <t>{saudacao} Volto com uma única observação, não com uma oferta: {valor} Vocês mantêm a relação e o serviço; nós entramos só na parte operacional. Se fizer sentido, façam uma triagem connosco: a página está pronta. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10753,17 +10753,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>D7: pergunta sim ou não</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho}. You bring in the demand; we work on the layer after the lead. The journey of one of your typical clients: {percurso}. I'm not assuming a problem; the question I'd validate: {pergunta} {isca} Companies in the US and China already work this way; in Romania, 5% of companies do (Eurostat, 2025). If not, run a triage with us: I've prepared a page (Micro System Print) with what I'd validate and a quick win you can apply right away, and we validate it together. I'll come prepared.</t>
+          <t>{saudacao} Uma pergunta simples, para não vos ocupar: o passo depois do lead já está resolvido de ponta a ponta nos vossos clientes, ou vale a pena validarmos o mapa juntos? Um sim ou um não chega. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10775,17 +10775,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>D4: observação nova</t>
+          <t>D12: fecho limpo</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Back with a single observation, not an offer: {valor} You keep the relationship and the service; we only step into the operational side. If it makes sense, run a triage with us: the page is ready. I'll come prepared.</t>
+          <t>{saudacao} Fecho o assunto por agora. Deixo-vos o Micro System Print; se este ponto se tornar prioridade para vocês ou para um cliente, validamos o mapa juntos. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10797,17 +10797,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>D7: pergunta sim ou não</t>
+          <t>Triagem (quando respondem, com o Micro System Print)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} One simple question, so I don't take your time: is the step after the lead already solved end to end for your clients, or is it worth validating the map together? A yes or a no is enough. I'll come prepared.</t>
+          <t>{saudacao} Obrigado pela resposta. Envio o Micro System Print de uma página: o percurso de um cliente típico vosso, o passo marcado «a validar» e o fluxo que proporia, com dono, regra e passagem a uma pessoa. Não afirmo que existe um problema: é a primeira coisa que validaria. Fazemos a triagem juntos, numa conversa curta em que eu conduzo as perguntas, sem formulários. Se o mapa se confirmar, implementamos 3 soluções rápidas, sem custo, na vossa operação, para verem como trabalhamos; o passo seguinte é a Auditoria de Sistemas com IA, creditada na implementação, em vocês ou num cliente. Se não se confirmar, a página fica como referência. Quando vos dá jeito? Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10819,17 +10819,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>D12: fecho limpo</t>
+          <t>Parceria (antes de aplicar os 3 quick wins: incentivo primeiro)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Closing this for now. I'll leave the Micro System Print with you; if this point becomes a priority for you or for a client, we validate the map together. I'll come prepared.</t>
+          <t>{saudacao} Antes de aplicarmos as 3 soluções, quero mostrar-vos o que podem ganhar se continuarmos a trabalhar juntos. Quando um cliente vosso encravar depois do lead e nos apresentarem, com o acordo dele, vocês mantêm o cliente e o serviço. Se chegarmos a trabalhar com ele, recebem 15% do valor da implementação e depois 5% de 3 em 3 meses, enquanto trabalharmos com ele. O valor depende do cliente: quanto maior a empresa, maior a implementação, e maior a vossa parte. Em troca pedimos três coisas, por esta ordem: no dia em que as 3 soluções ficam a funcionar, um primeiro testemunho online e uma recomendação, como agradecimento; depois, recomendações boca a boca; depois, uma menção por mês nos vossos conteúdos. Se vos parecer justo, envio a proposta escrita para assinar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10841,17 +10841,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Triagem (quando respondem, com o Micro System Print)</t>
+          <t>Testemunho (no dia em que os 3 quick wins ficam a funcionar)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Thanks for getting back to me. I'm sending the one-page Micro System Print: the journey of one of your typical clients, the step marked "to validate" and the flow I'd propose, with an owner, a rule and a human handoff. I'm not claiming there is a problem: it's the first thing I would validate. We run the triage together, in a short call where I lead the questions, no forms. If the map holds, we implement 3 quick wins at no cost in your own operation so you see how we work; the next step is the AI Systems Audit, credited against implementation, for you or for a client. If it doesn't hold, the page stays as a reference. When suits you? I'll come prepared.</t>
+          <t>{saudacao} As 3 soluções estão a funcionar desde hoje na vossa equipa. Obrigado pela confiança. Como combinámos, se estiverem satisfeitos, um primeiro testemunho online significava muito para nós: um post com @pachecostudiospt, nas vossas palavras, sobre o que mudou, e uma recomendação. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10868,144 +10868,144 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Parceria (depois dos 3 quick wins)</t>
+          <t>D0: DM 1</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Glad the 3 quick wins are already working for your team. I'd like to propose a simple partnership, starting with the part that matters to you: when one of your clients gets stuck after the lead, introduce us, with their consent. You keep the client and the service. If we end up working with that client, you get 15% of the implementation value and then 5% every 3 months for as long as we work with them. The value depends on the client: a bigger company means a bigger implementation, and a bigger share for you. If that feels fair, I'll send the written proposal with the simple rules: a testimonial from you and one post a month about us, tagging @pachecostudiospt. I'll come prepared.</t>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I saw {gancho}. You bring in the demand; we work on the layer after the lead. The journey of one of your typical clients: {percurso}. I'm not assuming a problem; the question I'd validate: {pergunta} {isca} Companies in the US and China already work this way; in Romania, 5% of companies do (Eurostat, 2025). If not, run a triage with us: I've prepared a page (Micro System Print) with what I'd validate and a quick win you can apply right away, and we validate it together. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>D4: observação nova</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Punctul despre {tema} mi se pare esențial. În operațiunile pe care le analizez, întrebarea care schimbă cel mai mult este: {pergunta}</t>
+          <t>{saudacao} Back with a single observation, not an offer: {valor} You keep the relationship and the service; we only step into the operational side. If it makes sense, run a triage with us: the page is ready. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>D7: pergunta sim ou não</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Bună observație. Aș adăuga un detaliu din practică: {valor}</t>
+          <t>{saudacao} One simple question, so I don't take your time: is the step after the lead already solved end to end for your clients, or is it worth validating the map together? A yes or a no is enough. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>D12: fecho limpo</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>O întrebare sinceră pentru cei care au trecut prin asta: {pergunta}</t>
+          <t>{saudacao} Closing this for now. I'll leave the Micro System Print with you; if this point becomes a priority for you or for a client, we validate the map together. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>Triagem (quando respondem, com o Micro System Print)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am comentat în ultimele săptămâni la postările voastre despre {tema}. Lucrez pe sisteme cu AI pentru operațiuni: unde stă contextul, cine răspunde de pasul următor și unde decide un om. Cred că publicul vostru ar găsi util un subiect ca acesta: {gancho}, ca articol, workshop scurt sau discuție la un eveniment. Ați fi deschis la o întâlnire scurtă? Voi fi pregătit.</t>
+          <t>{saudacao} Thanks for getting back to me. I'm sending the one-page Micro System Print: the journey of one of your typical clients, the step marked "to validate" and the flow I'd propose, with an owner, a rule and a human handoff. I'm not claiming there is a problem: it's the first thing I would validate. We run the triage together, in a short call where I lead the questions, no forms. If the map holds, we implement 3 quick wins at no cost in your own operation so you see how we work; the next step is the AI Systems Audit, credited against implementation, for you or for a client. If it doesn't hold, the page stays as a reference. When suits you? I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>D4: observação nova</t>
+          <t>Parceria (antes de aplicar os 3 quick wins: incentivo primeiro)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Revin cu propunerea de subiect, acum mai concretă: {valor} Mă adaptez formatului care vă ajută cel mai mult. Voi fi pregătit.</t>
+          <t>{saudacao} Before we apply the 3 quick wins, I want to show you what you can earn if we keep working together. When one of your clients gets stuck after the lead and you introduce us, with their consent, you keep the client and the service. If we end up working with them, you get 15% of the implementation value and then 5% every 3 months for as long as we work with them. The value depends on the client: the bigger the company, the bigger the implementation, and the bigger your share. In return we ask for three things, in this order: on the day the 3 quick wins go live, a first online testimonial and a recommendation, as a thank-you; then word-of-mouth recommendations; then one mention a month in your content. If that feels fair, I'll send the written proposal to sign. I'll come prepared.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Página / comunidade B2B</t>
+          <t>PME / parceiro de indicação</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>Testemunho (no dia em que os 3 quick wins ficam a funcionar)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>O ponto sobre {tema} parece-me essencial. Nas operações que analiso, a pergunta que mais muda o resultado é: {pergunta}</t>
+          <t>{saudacao} The 3 quick wins are live in your team as of today. Thank you for the trust. As agreed, if you're happy, a first online testimonial would mean a lot to us: a post tagging @pachecostudiospt, in your own words, about what changed, plus a recommendation. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -11017,17 +11017,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>Comentário: ponto</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Boa observação. Acrescentava um detalhe da prática: {valor}</t>
+          <t>Punctul despre {tema} mi se pare esențial. În operațiunile pe care le analizez, întrebarea care schimbă cel mai mult este: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -11039,17 +11039,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>Comentário: acréscimo</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Uma pergunta sincera para quem já passou por isto: {pergunta}</t>
+          <t>Bună observație. Aș adăuga un detaliu din practică: {valor}</t>
         </is>
       </c>
     </row>
@@ -11061,17 +11061,17 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>Comentário: pergunta</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Tenho comentado nas vossas publicações sobre {tema}. Trabalho em sistemas com IA para operações: onde fica o contexto, quem é dono do próximo passo e onde decide uma pessoa. Acho que a vossa audiência ia achar útil um tema como este: {gancho}, em artigo, workshop curto ou conversa num evento. Estariam abertos a uma reunião curta? Vou estar preparado.</t>
+          <t>O întrebare sinceră pentru cei care au trecut prin asta: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -11083,17 +11083,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>D4: observação nova</t>
+          <t>D0: DM 1</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Volto à proposta de tema, agora mais concreta: {valor} Adapto-me ao formato que mais vos ajudar. Vou estar preparado.</t>
+          <t>{saudacao} Sunt Tomás, de la Pacheco Studios, din Iași. Am comentat în ultimele săptămâni la postările voastre despre {tema}. Lucrez pe sisteme cu AI pentru operațiuni: unde stă contextul, cine răspunde de pasul următor și unde decide un om. Cred că publicul vostru ar găsi util un subiect ca acesta: {gancho}, ca articol, workshop scurt sau discuție la un eveniment. Ați fi deschis la o întâlnire scurtă? Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -11105,17 +11105,17 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Comentário: ponto</t>
+          <t>D4: observação nova</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>The point about {tema} is key. In the operations I map, the question that changes the most is: {pergunta}</t>
+          <t>{saudacao} Revin cu propunerea de subiect, acum mai concretă: {valor} Mă adaptez formatului care vă ajută cel mai mult. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -11127,17 +11127,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Comentário: acréscimo</t>
+          <t>Comentário: ponto</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Good point. One detail from practice I'd add: {valor}</t>
+          <t>O ponto sobre {tema} parece-me essencial. Nas operações que analiso, a pergunta que mais muda o resultado é: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -11149,17 +11149,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Comentário: pergunta</t>
+          <t>Comentário: acréscimo</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>An honest question for anyone who's been through this: {pergunta}</t>
+          <t>Boa observação. Acrescentava um detalhe da prática: {valor}</t>
         </is>
       </c>
     </row>
@@ -11171,17 +11171,17 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>D0: DM 1</t>
+          <t>Comentário: pergunta</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} I'm Tomás from Pacheco Studios. I've been commenting on your posts about {tema}. I work on AI systems for operations: where context lives, who owns the next step and where a human decides. I think your audience would find a topic like this useful: {gancho}, as an article, a short workshop or a talk at an event. Would you be open to a short meeting? I'll come prepared.</t>
+          <t>Uma pergunta sincera para quem já passou por isto: {pergunta}</t>
         </is>
       </c>
     </row>
@@ -11193,15 +11193,147 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>D0: DM 1</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>{saudacao} Sou o Tomás, da Pacheco Studios. Tenho comentado nas vossas publicações sobre {tema}. Trabalho em sistemas com IA para operações: onde fica o contexto, quem é dono do próximo passo e onde decide uma pessoa. Acho que a vossa audiência ia achar útil um tema como este: {gancho}, em artigo, workshop curto ou conversa num evento. Estariam abertos a uma reunião curta? Vou estar preparado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>D4: observação nova</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>{saudacao} Volto à proposta de tema, agora mais concreta: {valor} Adapto-me ao formato que mais vos ajudar. Vou estar preparado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
           <t>en</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Comentário: ponto</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>The point about {tema} is key. In the operations I map, the question that changes the most is: {pergunta}</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Comentário: acréscimo</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Good point. One detail from practice I'd add: {valor}</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Comentário: pergunta</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>An honest question for anyone who's been through this: {pergunta}</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>D0: DM 1</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>{saudacao} I'm Tomás from Pacheco Studios. I've been commenting on your posts about {tema}. I work on AI systems for operations: where context lives, who owns the next step and where a human decides. I think your audience would find a topic like this useful: {gancho}, as an article, a short workshop or a talk at an event. Would you be open to a short meeting? I'll come prepared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Página / comunidade B2B</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>D4: observação nova</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>{saudacao} Following up on the topic idea, now more concrete: {valor} Happy to fit whatever format helps you most. I'll come prepared.</t>
         </is>

</xml_diff>

<commit_message>
Instagram: base dos 5 % trimestrais confirmada (5 % dos nossos ganhos com a empresa, no fim de cada trimestre)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bCka4TNe6PKPBEx4M62DX
</commit_message>
<xml_diff>
--- a/research/instagram/prospecao-instagram.xlsx
+++ b/research/instagram/prospecao-instagram.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% de 3 em 3 meses; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
+          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% de 3 em 3 meses; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
+          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
         </is>
       </c>
       <c r="O3" s="2" t="n">
@@ -974,7 +974,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% de 3 em 3 meses; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
+          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
         </is>
       </c>
       <c r="O4" s="2" t="n">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% de 3 em 3 meses; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
+          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
         </is>
       </c>
       <c r="O5" s="2" t="n">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O7" s="2" t="n">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O8" s="2" t="n">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O9" s="2" t="n">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O10" s="2" t="n">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O11" s="2" t="n">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="O12" s="2" t="n">
@@ -9593,7 +9593,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% de 3 em 3 meses; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
+          <t>Triagem conduzida por nós (print + validação) → 3 quick wins → Auditoria de Sistemas com IA; parceria apresentada antes de aplicar os quick wins (incentivo primeiro: 15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; depois proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês nos conteúdos.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -9667,7 +9667,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% de 3 em 3 meses; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
+          <t>Triagem conduzida por nós → 3 quick wins → auditoria na operação deles ou de um cliente; parceria antes de aplicar os quick wins (15% da implementação + 5% dos nossos ganhos com o indicado no fim de cada trimestre; proposta assinada); contrapartida por ordem: testemunho online e recomendação no dia em que os quick wins funcionam, boca a boca, 1 menção por mês.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Înainte să aplicăm cele 3 soluții, vreau să-ți arăt ce poți câștiga dacă lucrăm și mai departe împreună. Când ne prezinți o afacere care se blochează în același loc, cu acordul ei, și ajungem să lucrăm cu ea, primești 15% din valoarea implementării și apoi 5% la fiecare 3 luni, cât timp lucrăm cu ea. Valoarea depinde de afacere: cu cât firma e mai mare, cu atât implementarea e mai mare, și la fel partea ta. În schimb îți cerem trei lucruri, în ordinea asta: în ziua în care cele 3 soluții funcționează, un prim testimonial online și o recomandare, ca mulțumire; apoi recomandări din gură în gură; apoi o mențiune pe lună în conținutul tău. Dacă ți se pare corect, îți trimit propunerea scrisă, de semnat. Voi fi pregătit.</t>
+          <t>{saudacao} Înainte să aplicăm cele 3 soluții, vreau să-ți arăt ce poți câștiga dacă lucrăm și mai departe împreună. Când ne prezinți o afacere care se blochează în același loc, cu acordul ei, și ajungem să lucrăm cu ea, primești 15% din valoarea implementării și apoi 5% din ce câștigăm noi cu ea, plătit la sfârșitul fiecărui trimestru, cât timp lucrăm cu ea. Valoarea depinde de afacere: cu cât firma e mai mare, cu atât implementarea e mai mare, și la fel partea ta. În schimb îți cerem trei lucruri, în ordinea asta: în ziua în care cele 3 soluții funcționează, un prim testimonial online și o recomandare, ca mulțumire; apoi recomandări din gură în gură; apoi o mențiune pe lună în conținutul tău. Dacă ți se pare corect, îți trimit propunerea scrisă, de semnat. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10037,7 +10037,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Antes de aplicarmos as 3 soluções, quero mostrar-te o que podes ganhar se continuarmos a trabalhar juntos. Quando nos apresentares um negócio que encrava no mesmo sítio, com o acordo dele, e chegarmos a trabalhar com ele, recebes 15% do valor da implementação e depois 5% de 3 em 3 meses, enquanto trabalharmos com ele. O valor depende do negócio: quanto maior a empresa, maior a implementação, e maior a tua parte. Em troca pedimos três coisas, por esta ordem: no dia em que as 3 soluções ficam a funcionar, um primeiro testemunho online e uma recomendação, como agradecimento; depois, recomendações boca a boca; depois, uma menção por mês nos teus conteúdos. Se te parecer justo, envio a proposta escrita para assinar. Vou estar preparado.</t>
+          <t>{saudacao} Antes de aplicarmos as 3 soluções, quero mostrar-te o que podes ganhar se continuarmos a trabalhar juntos. Quando nos apresentares um negócio que encrava no mesmo sítio, com o acordo dele, e chegarmos a trabalhar com ele, recebes 15% do valor da implementação e depois 5% do que ganhamos com ele, pago no fim de cada trimestre, enquanto trabalharmos com ele. O valor depende do negócio: quanto maior a empresa, maior a implementação, e maior a tua parte. Em troca pedimos três coisas, por esta ordem: no dia em que as 3 soluções ficam a funcionar, um primeiro testemunho online e uma recomendação, como agradecimento; depois, recomendações boca a boca; depois, uma menção por mês nos teus conteúdos. Se te parecer justo, envio a proposta escrita para assinar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10191,7 +10191,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Before we apply the 3 quick wins, I want to show you what you can earn if we keep working together. When you introduce us to a business stuck in the same place, with their consent, and we end up working with them, you get 15% of the implementation value and then 5% every 3 months for as long as we work with them. The value depends on the business: the bigger the company, the bigger the implementation, and the bigger your share. In return we ask for three things, in this order: on the day the 3 quick wins go live, a first online testimonial and a recommendation, as a thank-you; then word-of-mouth recommendations; then one mention a month in your content. If that feels fair, I'll send the written proposal to sign. I'll come prepared.</t>
+          <t>{saudacao} Before we apply the 3 quick wins, I want to show you what you can earn if we keep working together. When you introduce us to a business stuck in the same place, with their consent, and we end up working with them, you get 15% of the implementation value and then 5% of what we earn with them, paid at the end of every quarter, for as long as we work with them. The value depends on the business: the bigger the company, the bigger the implementation, and the bigger your share. In return we ask for three things, in this order: on the day the 3 quick wins go live, a first online testimonial and a recommendation, as a thank-you; then word-of-mouth recommendations; then one mention a month in your content. If that feels fair, I'll send the written proposal to sign. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -10675,7 +10675,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Înainte să aplicăm cele 3 soluții, vreau să vă arăt ce puteți câștiga dacă lucrăm și mai departe împreună. Când un client de-al vostru se blochează după lead și ne faceți o introducere, cu acordul lui, voi păstrați clientul și serviciul. Dacă ajungem să lucrăm cu el, primiți 15% din valoarea implementării și apoi 5% la fiecare 3 luni, cât timp lucrăm cu el. Valoarea depinde de client: cu cât firma e mai mare, cu atât implementarea e mai mare, și la fel partea voastră. În schimb vă cerem trei lucruri, în ordinea asta: în ziua în care cele 3 soluții funcționează, un prim testimonial online și o recomandare, ca mulțumire; apoi recomandări din gură în gură; apoi o mențiune pe lună în conținutul vostru. Dacă vi se pare corect, vă trimit propunerea scrisă, de semnat. Voi fi pregătit.</t>
+          <t>{saudacao} Înainte să aplicăm cele 3 soluții, vreau să vă arăt ce puteți câștiga dacă lucrăm și mai departe împreună. Când un client de-al vostru se blochează după lead și ne faceți o introducere, cu acordul lui, voi păstrați clientul și serviciul. Dacă ajungem să lucrăm cu el, primiți 15% din valoarea implementării și apoi 5% din ce câștigăm noi cu el, plătit la sfârșitul fiecărui trimestru, cât timp lucrăm cu el. Valoarea depinde de client: cu cât firma e mai mare, cu atât implementarea e mai mare, și la fel partea voastră. În schimb vă cerem trei lucruri, în ordinea asta: în ziua în care cele 3 soluții funcționează, un prim testimonial online și o recomandare, ca mulțumire; apoi recomandări din gură în gură; apoi o mențiune pe lună în conținutul vostru. Dacă vi se pare corect, vă trimit propunerea scrisă, de semnat. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10829,7 +10829,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Antes de aplicarmos as 3 soluções, quero mostrar-vos o que podem ganhar se continuarmos a trabalhar juntos. Quando um cliente vosso encravar depois do lead e nos apresentarem, com o acordo dele, vocês mantêm o cliente e o serviço. Se chegarmos a trabalhar com ele, recebem 15% do valor da implementação e depois 5% de 3 em 3 meses, enquanto trabalharmos com ele. O valor depende do cliente: quanto maior a empresa, maior a implementação, e maior a vossa parte. Em troca pedimos três coisas, por esta ordem: no dia em que as 3 soluções ficam a funcionar, um primeiro testemunho online e uma recomendação, como agradecimento; depois, recomendações boca a boca; depois, uma menção por mês nos vossos conteúdos. Se vos parecer justo, envio a proposta escrita para assinar. Vou estar preparado.</t>
+          <t>{saudacao} Antes de aplicarmos as 3 soluções, quero mostrar-vos o que podem ganhar se continuarmos a trabalhar juntos. Quando um cliente vosso encravar depois do lead e nos apresentarem, com o acordo dele, vocês mantêm o cliente e o serviço. Se chegarmos a trabalhar com ele, recebem 15% do valor da implementação e depois 5% do que ganhamos com ele, pago no fim de cada trimestre, enquanto trabalharmos com ele. O valor depende do cliente: quanto maior a empresa, maior a implementação, e maior a vossa parte. Em troca pedimos três coisas, por esta ordem: no dia em que as 3 soluções ficam a funcionar, um primeiro testemunho online e uma recomendação, como agradecimento; depois, recomendações boca a boca; depois, uma menção por mês nos vossos conteúdos. Se vos parecer justo, envio a proposta escrita para assinar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Before we apply the 3 quick wins, I want to show you what you can earn if we keep working together. When one of your clients gets stuck after the lead and you introduce us, with their consent, you keep the client and the service. If we end up working with them, you get 15% of the implementation value and then 5% every 3 months for as long as we work with them. The value depends on the client: the bigger the company, the bigger the implementation, and the bigger your share. In return we ask for three things, in this order: on the day the 3 quick wins go live, a first online testimonial and a recommendation, as a thank-you; then word-of-mouth recommendations; then one mention a month in your content. If that feels fair, I'll send the written proposal to sign. I'll come prepared.</t>
+          <t>{saudacao} Before we apply the 3 quick wins, I want to show you what you can earn if we keep working together. When one of your clients gets stuck after the lead and you introduce us, with their consent, you keep the client and the service. If we end up working with them, you get 15% of the implementation value and then 5% of what we earn with them, paid at the end of every quarter, for as long as we work with them. The value depends on the client: the bigger the company, the bigger the implementation, and the bigger your share. In return we ask for three things, in this order: on the day the 3 quick wins go live, a first online testimonial and a recommendation, as a thank-you; then word-of-mouth recommendations; then one mention a month in your content. If that feels fair, I'll send the written proposal to sign. I'll come prepared.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Instagram: quick wins dos parceiros em 9 áreas amplas e testemunho sem guião (decisão de 18h31)
Mensagens «Parceria» e «Testemunho» (RO/PT/EN), COMISSAO-PARCEIROS.md, LEIA-ME,
guião da mesa e exemplos do brief sem fichas Google nem cartazes de avaliações.
Os 19 DMs do lote 1 ficam iguais.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bCka4TNe6PKPBEx4M62DX
</commit_message>
<xml_diff>
--- a/research/instagram/prospecao-instagram.xlsx
+++ b/research/instagram/prospecao-instagram.xlsx
@@ -9883,7 +9883,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Înainte să aplicăm cele 3 soluții, vreau să-ți arăt ce poți câștiga dacă lucrăm și mai departe împreună. Când ne prezinți o afacere care se blochează în același loc, cu acordul ei, și ajungem să lucrăm cu ea, primești 15% din valoarea implementării și apoi 5% din ce câștigăm noi cu ea, plătit la sfârșitul fiecărui trimestru, cât timp lucrăm cu ea. Valoarea depinde de afacere: cu cât firma e mai mare, cu atât implementarea e mai mare, și la fel partea ta. În schimb îți cerem trei lucruri, în ordinea asta: în ziua în care cele 3 soluții funcționează, un prim testimonial online și o recomandare, ca mulțumire; apoi recomandări din gură în gură; apoi o mențiune pe lună în conținutul tău. Dacă ți se pare corect, îți trimit propunerea scrisă, de semnat. Voi fi pregătit.</t>
+          <t>{saudacao} Înainte să aplicăm cele 3 soluții, vreau să-ți arăt ce poți câștiga dacă lucrăm și mai departe împreună. Soluțiile le alegem din 9 zone largi, de la clienți și facturi la răspuns automat și recenzii, după situația ta. Când ne prezinți o afacere care se blochează în același loc, cu acordul ei, și ajungem să lucrăm cu ea, primești 15% din valoarea implementării și apoi 5% din ce câștigăm noi cu ea, plătit la sfârșitul fiecărui trimestru, cât timp lucrăm cu ea. Cu cât afacerea e mai mare, cu atât implementarea și partea ta sunt mai mari. În schimb îți cerem trei lucruri, în ordinea asta: în ziua în care cele 3 soluții funcționează, un prim testimonial online și o recomandare, ca mulțumire; apoi recomandări din gură în gură; apoi o mențiune pe lună în conținutul tău. Dacă ți se pare corect, îți trimit propunerea scrisă, de semnat. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -9905,7 +9905,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Cele 3 soluții funcționează de azi. Mulțumesc pentru încredere. Cum am vorbit, dacă ești mulțumit, un prim testimonial online ar însemna mult pentru noi: o postare sau un story cu @pachecostudiospt, în cuvintele tale, despre ce s-a schimbat, și o recomandare. Voi fi pregătit.</t>
+          <t>{saudacao} Cele 3 soluții funcționează de azi. Mulțumesc pentru încredere. Cum am vorbit, dacă ești mulțumit, un prim testimonial online și o recomandare ar însemna mult pentru noi. Fără scenariu și fără text de la noi: vorbește despre noi cu cuvintele tale, despre ce ai văzut funcționând, unde vrei, cu @pachecostudiospt. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10037,7 +10037,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Antes de aplicarmos as 3 soluções, quero mostrar-te o que podes ganhar se continuarmos a trabalhar juntos. Quando nos apresentares um negócio que encrava no mesmo sítio, com o acordo dele, e chegarmos a trabalhar com ele, recebes 15% do valor da implementação e depois 5% do que ganhamos com ele, pago no fim de cada trimestre, enquanto trabalharmos com ele. O valor depende do negócio: quanto maior a empresa, maior a implementação, e maior a tua parte. Em troca pedimos três coisas, por esta ordem: no dia em que as 3 soluções ficam a funcionar, um primeiro testemunho online e uma recomendação, como agradecimento; depois, recomendações boca a boca; depois, uma menção por mês nos teus conteúdos. Se te parecer justo, envio a proposta escrita para assinar. Vou estar preparado.</t>
+          <t>{saudacao} Antes de aplicarmos as 3 soluções, quero mostrar-te o que podes ganhar se continuarmos a trabalhar juntos. As soluções escolhem-se em 9 áreas amplas, de clientes e faturas a atendimento automático e avaliações, conforme a tua situação. Quando nos apresentares um negócio que encrava no mesmo sítio, com o acordo dele, e chegarmos a trabalhar com ele, recebes 15% do valor da implementação e depois 5% do que ganhamos com ele, pago no fim de cada trimestre, enquanto trabalharmos com ele. Quanto maior o negócio, maior a implementação e a tua parte. Em troca pedimos três coisas, por esta ordem: no dia em que as 3 soluções ficam a funcionar, um primeiro testemunho online e uma recomendação, como agradecimento; depois, recomendações boca a boca; depois, uma menção por mês nos teus conteúdos. Se te parecer justo, envio a proposta escrita para assinar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10059,7 +10059,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} As 3 soluções estão a funcionar desde hoje. Obrigado pela confiança. Como combinámos, se estiveres satisfeito, um primeiro testemunho online significava muito para nós: um post ou story com @pachecostudiospt, nas tuas palavras, sobre o que mudou, e uma recomendação. Vou estar preparado.</t>
+          <t>{saudacao} As 3 soluções estão a funcionar desde hoje. Obrigado pela confiança. Como combinámos, se estiveres satisfeito, um primeiro testemunho online e uma recomendação significavam muito para nós. Sem guião e sem texto nosso: fala de nós com as tuas palavras, sobre o que viste a funcionar, onde quiseres, com @pachecostudiospt. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10191,7 +10191,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Before we apply the 3 quick wins, I want to show you what you can earn if we keep working together. When you introduce us to a business stuck in the same place, with their consent, and we end up working with them, you get 15% of the implementation value and then 5% of what we earn with them, paid at the end of every quarter, for as long as we work with them. The value depends on the business: the bigger the company, the bigger the implementation, and the bigger your share. In return we ask for three things, in this order: on the day the 3 quick wins go live, a first online testimonial and a recommendation, as a thank-you; then word-of-mouth recommendations; then one mention a month in your content. If that feels fair, I'll send the written proposal to sign. I'll come prepared.</t>
+          <t>{saudacao} Before we apply the 3 quick wins, I want to show you what you can earn if we keep working together. We pick them from 9 broad areas, from clients and invoices to automatic replies and reviews, depending on your situation. When you introduce us to a business stuck in the same place, with their consent, and we end up working with them, you get 15% of the implementation value and then 5% of what we earn with them, paid at the end of every quarter, for as long as we work with them. The bigger the business, the bigger the implementation and your share. In return we ask for three things, in this order: on the day the 3 quick wins go live, a first online testimonial and a recommendation, as a thank-you; then word-of-mouth recommendations; then one mention a month in your content. If that feels fair, I'll send the written proposal to sign. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -10213,7 +10213,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} The 3 quick wins are live as of today. Thank you for the trust. As agreed, if you're happy, a first online testimonial would mean a lot to us: a post or story tagging @pachecostudiospt, in your own words, about what changed, plus a recommendation. I'll come prepared.</t>
+          <t>{saudacao} The 3 quick wins are live as of today. Thank you for the trust. As agreed, if you're happy, a first online testimonial and a recommendation would mean a lot to us. No script and no text from us: talk about us in your own words, about what you saw working, wherever you like, tagging @pachecostudiospt. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -10675,7 +10675,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Înainte să aplicăm cele 3 soluții, vreau să vă arăt ce puteți câștiga dacă lucrăm și mai departe împreună. Când un client de-al vostru se blochează după lead și ne faceți o introducere, cu acordul lui, voi păstrați clientul și serviciul. Dacă ajungem să lucrăm cu el, primiți 15% din valoarea implementării și apoi 5% din ce câștigăm noi cu el, plătit la sfârșitul fiecărui trimestru, cât timp lucrăm cu el. Valoarea depinde de client: cu cât firma e mai mare, cu atât implementarea e mai mare, și la fel partea voastră. În schimb vă cerem trei lucruri, în ordinea asta: în ziua în care cele 3 soluții funcționează, un prim testimonial online și o recomandare, ca mulțumire; apoi recomandări din gură în gură; apoi o mențiune pe lună în conținutul vostru. Dacă vi se pare corect, vă trimit propunerea scrisă, de semnat. Voi fi pregătit.</t>
+          <t>{saudacao} Înainte să aplicăm cele 3 soluții, vreau să vă arăt ce puteți câștiga dacă lucrăm și mai departe împreună. Soluțiile le alegem din 9 zone largi, de la clienți și facturi la răspuns automat și recenzii, după situația voastră. Când un client de-al vostru se blochează după lead și ne faceți o introducere, cu acordul lui, voi păstrați clientul și serviciul. Dacă ajungem să lucrăm cu el, primiți 15% din valoarea implementării și apoi 5% din ce câștigăm noi cu el, plătit la sfârșitul fiecărui trimestru, cât timp lucrăm cu el. Cu cât clientul e mai mare, cu atât implementarea și partea voastră sunt mai mari. În schimb vă cerem trei lucruri, în ordinea asta: în ziua în care cele 3 soluții funcționează, un prim testimonial online și o recomandare, ca mulțumire; apoi recomandări din gură în gură; apoi o mențiune pe lună în conținutul vostru. Dacă vi se pare corect, vă trimit propunerea scrisă, de semnat. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10697,7 +10697,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Cele 3 soluții funcționează de azi în echipa voastră. Mulțumesc pentru încredere. Cum am vorbit, dacă sunteți mulțumiți, un prim testimonial online ar însemna mult pentru noi: o postare cu @pachecostudiospt, în cuvintele voastre, despre ce s-a schimbat, și o recomandare. Voi fi pregătit.</t>
+          <t>{saudacao} Cele 3 soluții funcționează de azi în echipa voastră. Mulțumesc pentru încredere. Cum am vorbit, dacă sunteți mulțumiți, un prim testimonial online și o recomandare ar însemna mult pentru noi. Fără scenariu și fără text de la noi: vorbiți despre noi cu cuvintele voastre, despre ce ați văzut funcționând, cu @pachecostudiospt. Voi fi pregătit.</t>
         </is>
       </c>
     </row>
@@ -10829,7 +10829,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Antes de aplicarmos as 3 soluções, quero mostrar-vos o que podem ganhar se continuarmos a trabalhar juntos. Quando um cliente vosso encravar depois do lead e nos apresentarem, com o acordo dele, vocês mantêm o cliente e o serviço. Se chegarmos a trabalhar com ele, recebem 15% do valor da implementação e depois 5% do que ganhamos com ele, pago no fim de cada trimestre, enquanto trabalharmos com ele. O valor depende do cliente: quanto maior a empresa, maior a implementação, e maior a vossa parte. Em troca pedimos três coisas, por esta ordem: no dia em que as 3 soluções ficam a funcionar, um primeiro testemunho online e uma recomendação, como agradecimento; depois, recomendações boca a boca; depois, uma menção por mês nos vossos conteúdos. Se vos parecer justo, envio a proposta escrita para assinar. Vou estar preparado.</t>
+          <t>{saudacao} Antes de aplicarmos as 3 soluções, quero mostrar-vos o que podem ganhar se continuarmos a trabalhar juntos. As soluções escolhem-se em 9 áreas amplas, de clientes e faturas a atendimento automático e avaliações, conforme a vossa situação. Quando um cliente vosso encravar depois do lead e nos apresentarem, com o acordo dele, vocês mantêm o cliente e o serviço. Se chegarmos a trabalhar com ele, recebem 15% do valor da implementação e depois 5% do que ganhamos com ele, pago no fim de cada trimestre, enquanto trabalharmos com ele. Quanto maior o cliente, maior a implementação e a vossa parte. Em troca pedimos três coisas, por esta ordem: no dia em que as 3 soluções ficam a funcionar, um primeiro testemunho online e uma recomendação, como agradecimento; depois, recomendações boca a boca; depois, uma menção por mês nos vossos conteúdos. Se vos parecer justo, envio a proposta escrita para assinar. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10851,7 +10851,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} As 3 soluções estão a funcionar desde hoje na vossa equipa. Obrigado pela confiança. Como combinámos, se estiverem satisfeitos, um primeiro testemunho online significava muito para nós: um post com @pachecostudiospt, nas vossas palavras, sobre o que mudou, e uma recomendação. Vou estar preparado.</t>
+          <t>{saudacao} As 3 soluções estão a funcionar desde hoje na vossa equipa. Obrigado pela confiança. Como combinámos, se estiverem satisfeitos, um primeiro testemunho online e uma recomendação significavam muito para nós. Sem guião e sem texto nosso: falem de nós com as vossas palavras, sobre o que viram a funcionar, com @pachecostudiospt. Vou estar preparado.</t>
         </is>
       </c>
     </row>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} Before we apply the 3 quick wins, I want to show you what you can earn if we keep working together. When one of your clients gets stuck after the lead and you introduce us, with their consent, you keep the client and the service. If we end up working with them, you get 15% of the implementation value and then 5% of what we earn with them, paid at the end of every quarter, for as long as we work with them. The value depends on the client: the bigger the company, the bigger the implementation, and the bigger your share. In return we ask for three things, in this order: on the day the 3 quick wins go live, a first online testimonial and a recommendation, as a thank-you; then word-of-mouth recommendations; then one mention a month in your content. If that feels fair, I'll send the written proposal to sign. I'll come prepared.</t>
+          <t>{saudacao} Before we apply the 3 quick wins, I want to show you what you can earn if we keep working together. We pick them from 9 broad areas, from clients and invoices to automatic replies and reviews, depending on your situation. When one of your clients gets stuck after the lead and you introduce us, with their consent, you keep the client and the service. If we end up working with them, you get 15% of the implementation value and then 5% of what we earn with them, paid at the end of every quarter, for as long as we work with them. The bigger the client, the bigger the implementation and your share. In return we ask for three things, in this order: on the day the 3 quick wins go live, a first online testimonial and a recommendation, as a thank-you; then word-of-mouth recommendations; then one mention a month in your content. If that feels fair, I'll send the written proposal to sign. I'll come prepared.</t>
         </is>
       </c>
     </row>
@@ -11005,7 +11005,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>{saudacao} The 3 quick wins are live in your team as of today. Thank you for the trust. As agreed, if you're happy, a first online testimonial would mean a lot to us: a post tagging @pachecostudiospt, in your own words, about what changed, plus a recommendation. I'll come prepared.</t>
+          <t>{saudacao} The 3 quick wins are live in your team as of today. Thank you for the trust. As agreed, if you're happy, a first online testimonial and a recommendation would mean a lot to us. No script and no text from us: talk about us in your own words, about what you saw working, tagging @pachecostudiospt. I'll come prepared.</t>
         </is>
       </c>
     </row>

</xml_diff>